<commit_message>
SPM-68: release and withdraw cases, October fixture dates, documentation
- AC12's release half, now that SPM-67 is on main: SPM-68-TC16 and TC17,
  and page tests for Release booking / Withdraw request, which call
  SPM-67's own route.
- Move every test date from September to October 2027: the app writes
  September as "Sept", so the expected "8 Sep 2027" strings were wrong.
- DOCUMENTATION.md: changelog entry for the test-first work and the
  contract it sets; Known Gaps note that flags still cannot be cleared.

The SPM-68 tests still fail by design until the code is built.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-68_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-68_Test_Cases.xlsx
@@ -23,6 +23,8 @@
     <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TC17" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -462,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -982,7 +984,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Requesting a replacement venue adds a pending request and leaves the flagged booking, the event's information and its status unchanged</t>
+          <t>Requesting a replacement venue adds a pending request and leaves the flagged booking on the event record, and the event's information and status unchanged</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1001,40 +1003,104 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC16</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Releasing a flagged booking from the Flagged Arrangements page asks first, takes it off the page, keeps it on the event record as Released and leaves the replacement request and the event unchanged</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>AC12, AC13, AC14</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TC17</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC17</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>A flagged venue request that is still pending is withdrawn, not released, from the Flagged Arrangements page</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>AC12, AC14</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Covered by</t>
         </is>
       </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC02
@@ -1042,22 +1108,22 @@
 SPM-68-TC04</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Each flagged arrangement shows the event, the arrangement, and why it was flagged (e.g. event date changed, attendance changed, venue attributes updated, venue setup or turnaround time changed, venue retired, venue blocked, equipment marked unavailable).</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC08
@@ -1065,42 +1131,42 @@
 SPM-68-TC11</t>
         </is>
       </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="31" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="31" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Given an event has more than one venue booking, when one of them is flagged, then only the flagged booking is listed.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="71.5" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="71.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC06
@@ -1109,65 +1175,65 @@
 SPM-68-TC09</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="44.5" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="44.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>For a flagged equipment reservation, the current availability result for the event's present dates and quantities is shown.</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC10
 SPM-68-TC11</t>
         </is>
       </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="44.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="44.5" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>AC6</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Given the arrangement still meets the event's requirements, when the Coordinator keeps it, then the flag is cleared and the arrangement is unchanged.</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC06
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>AC7</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC07
 SPM-68-TC08
@@ -1175,143 +1241,146 @@
 SPM-68-TC11</t>
         </is>
       </c>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="71.5" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="F30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="71.5" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>AC8</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>For flagged registrations, the number of attendees registered or on the waiting list is shown, with why they were flagged: the event's date or time changed (see: Update Event Information, SPM-62), or the registration capacity was lowered below the number registered or registration was turned off (see: Configure Event Registration, SPM-64).</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01
-SPM-68-TC12</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n"/>
-    </row>
-    <row r="30" ht="31" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>AC9</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC12</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n"/>
-    </row>
-    <row r="31" ht="17.5" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>AC10</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>Flagged registrations do not prevent confirmation.</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13</t>
+          <t>SPM-68-TC01
+SPM-68-TC12</t>
         </is>
       </c>
       <c r="F31" s="9" t="n"/>
     </row>
-    <row r="32" ht="58" customHeight="1">
+    <row r="32" ht="31" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC9</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
+          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC14</t>
+          <t>SPM-68-TC12</t>
         </is>
       </c>
       <c r="F32" s="9" t="n"/>
     </row>
-    <row r="33" ht="44.5" customHeight="1">
+    <row r="33" ht="17.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC10</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
+          <t>Flagged registrations do not prevent confirmation.</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC15</t>
+          <t>SPM-68-TC13</t>
         </is>
       </c>
       <c r="F33" s="9" t="n"/>
     </row>
-    <row r="34" ht="31" customHeight="1">
+    <row r="34" ht="58" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC11</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Replacing a venue does not change the event's own information or status.</t>
+          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC15</t>
+          <t>SPM-68-TC14</t>
         </is>
       </c>
       <c r="F34" s="9" t="n"/>
     </row>
-    <row r="35" ht="98.5" customHeight="1">
+    <row r="35" ht="44.5" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>AC14</t>
+          <t>AC12</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
         </is>
       </c>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC15
+SPM-68-TC16
+SPM-68-TC17</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="31" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>AC13</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Replacing a venue does not change the event's own information or status.</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC15
+SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="125.5" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>AC14</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC05
 SPM-68-TC06
@@ -1319,51 +1388,53 @@
 SPM-68-TC08
 SPM-68-TC10
 SPM-68-TC11
-SPM-68-TC15</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="44.5" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+SPM-68-TC15
+SPM-68-TC16
+SPM-68-TC17</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="44.5" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>AC15</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>A flagged venue booking or equipment reservation counts as outstanding and prevents confirmation until it is resolved (see: Track Outstanding Arrangements).</t>
         </is>
       </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC05
 SPM-68-TC06</t>
         </is>
       </c>
-      <c r="F36" s="9" t="n"/>
-    </row>
-    <row r="37" ht="31" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="F38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="31" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>AC16</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC02</t>
         </is>
       </c>
-      <c r="F37" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="35">
@@ -1372,16 +1443,19 @@
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="B38:D38"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="E31:F31"/>
     <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E31:F31"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B36:D36"/>
@@ -1396,12 +1470,9 @@
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E25:F25"/>
-    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B39:D39"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1419,6 +1490,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1477,7 +1550,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Venue Trouble Day' is in Planning, assigned to Daniel Tan, on 9 Sep 2027, 09:00-17:00, for 40 people in Theatre layout. It has two approved venue bookings, both flagged: SPM68 Closed Room, which Venue Staff marked unavailable for maintenance from 9 Sep 2027, 08:00 to 9 Sep 2027, 18:00; and SPM68 Retired Room, which has been retired. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Venue Trouble Day' is in Planning, assigned to Daniel Tan, on 9 Oct 2027, 09:00-17:00, for 40 people in Theatre layout. It has two approved venue bookings, both flagged: SPM68 Closed Room, which Venue Staff marked unavailable for maintenance from 9 Oct 2027, 08:00 to 9 Oct 2027, 18:00; and SPM68 Retired Room, which has been retired. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
         </is>
       </c>
     </row>
@@ -1505,8 +1578,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Venue Trouble Day (Planning), 9 Sep 2027, 09:00-17:00, 40 people, Theatre
-SPM68 Closed Room (Approved, flagged): unavailable for maintenance 9 Sep 2027, 08:00-18:00
+          <t>Event: SPM68 Venue Trouble Day (Planning), 9 Oct 2027, 09:00-17:00, 40 people, Theatre
+SPM68 Closed Room (Approved, flagged): unavailable for maintenance 9 Oct 2027, 08:00-18:00
 SPM68 Retired Room (Approved, flagged): retired</t>
         </is>
       </c>
@@ -1519,10 +1592,10 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: Two separate items are listed for 'SPM68 Venue Trouble Day'. The SPM68 Closed Room item shows 'Flagged because: the venue is unavailable during this booking', 'Suitability: Suitable' and 'Availability: Not available' with 'SPM68 Closed Room is unavailable at this time (maintenance, 9 Sep 2027, 08:00–18:00).' The SPM68 Retired Room item shows 'Flagged because: the venue has been retired' and 'Availability: Not available' with 'SPM68 Retired Room has been retired.'
-Step 2: The flag is NOT cleared. The message 'SPM68 Closed Room no longer meets this event's requirements: SPM68 Closed Room is unavailable at this time (maintenance, 9 Sep 2027, 08:00–18:00).' is shown in that item, and the item is still listed.
+          <t>Step 1: Two separate items are listed for 'SPM68 Venue Trouble Day'. The SPM68 Closed Room item shows 'Flagged because: the venue is unavailable during this booking', 'Suitability: Suitable' and 'Availability: Not available' with 'SPM68 Closed Room is unavailable at this time (maintenance, 9 Oct 2027, 08:00–18:00).' The SPM68 Retired Room item shows 'Flagged because: the venue has been retired' and 'Availability: Not available' with 'SPM68 Retired Room has been retired.'
+Step 2: The flag is NOT cleared. The message 'SPM68 Closed Room no longer meets this event's requirements: SPM68 Closed Room is unavailable at this time (maintenance, 9 Oct 2027, 08:00–18:00).' is shown in that item, and the item is still listed.
 Step 3: The flag is NOT cleared. The message 'SPM68 Retired Room no longer meets this event's requirements: SPM68 Retired Room has been retired.' is shown in that item, and the item is still listed.
-Step 5: Under 'Booking requests', SPM68 Closed Room and SPM68 Retired Room are both still listed as 'Approved' for 9 Sep 2027, 09:00–17:00. Neither was changed or cancelled.</t>
+Step 5: Under 'Booking requests', SPM68 Closed Room and SPM68 Retired Room are both still listed as 'Approved' for 9 Oct 2027, 09:00–17:00. Neither was changed or cancelled.</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1728,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Moved Date' is in Planning, assigned to Daniel Tan, for 40 people in Theatre layout. The event was moved to 14 Sep 2027, 09:00-17:00, but its approved booking at SPM68 Annex is still for 13 Sep 2027, 09:00-17:00 and is flagged because the date or time changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Moved Date' is in Planning, assigned to Daniel Tan, for 40 people in Theatre layout. The event was moved to 14 Oct 2027, 09:00-17:00, but its approved booking at SPM68 Annex is still for 13 Oct 2027, 09:00-17:00 and is flagged because the date or time changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
         </is>
       </c>
     </row>
@@ -1680,8 +1753,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Moved Date (Planning), now 14 Sep 2027, 09:00-17:00, 40 people, Theatre
-Venue booking: SPM68 Annex (Approved, flagged), 13 Sep 2027, 09:00-17:00</t>
+          <t>Event: SPM68 Moved Date (Planning), now 14 Oct 2027, 09:00-17:00, 40 people, Theatre
+Venue booking: SPM68 Annex (Approved, flagged), 13 Oct 2027, 09:00-17:00</t>
         </is>
       </c>
     </row>
@@ -1693,8 +1766,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'SPM68 Moved Date' item shows 'SPM68 Annex (SPM68-ANX)', '13 Sep 2027, 09:00–17:00', 'Flagged because: the date or time changed', 'Suitability: Suitable' and 'Availability: Not available' with 'The booking (13 Sep 2027, 09:00–17:00) does not cover the event's time (14 Sep 2027, 09:00–17:00).'
-Step 2: The flag is NOT cleared. The message 'SPM68 Annex no longer meets this event's requirements: The booking (13 Sep 2027, 09:00–17:00) does not cover the event's time (14 Sep 2027, 09:00–17:00).' is shown in the item, and the item is still listed with the booking still on 13 Sep 2027.</t>
+          <t>Step 1: The 'SPM68 Moved Date' item shows 'SPM68 Annex (SPM68-ANX)', '13 Oct 2027, 09:00–17:00', 'Flagged because: the date or time changed', 'Suitability: Suitable' and 'Availability: Not available' with 'The booking (13 Oct 2027, 09:00–17:00) does not cover the event's time (14 Oct 2027, 09:00–17:00).'
+Step 2: The flag is NOT cleared. The message 'SPM68 Annex no longer meets this event's requirements: The booking (13 Oct 2027, 09:00–17:00) does not cover the event's time (14 Oct 2027, 09:00–17:00).' is shown in the item, and the item is still listed with the booking still on 13 Oct 2027.</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1900,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Kit Recheck' is in Planning, assigned to Daniel Tan, on 15 Sep 2027, 09:00-17:00. Its reservation of 2 SPM68 Projector (Reserved; 4 in stock, none out of service, no other event holds any that day) is flagged because the date or time changed. Logged in as Daniel Tan.</t>
+          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Kit Recheck' is in Planning, assigned to Daniel Tan, on 15 Oct 2027, 09:00-17:00. Its reservation of 2 SPM68 Projector (Reserved; 4 in stock, none out of service, no other event holds any that day) is flagged because the date or time changed. Logged in as Daniel Tan.</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1928,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Kit Recheck (Planning), 15 Sep 2027, 09:00-17:00
+          <t>Event: SPM68 Kit Recheck (Planning), 15 Oct 2027, 09:00-17:00
 Equipment: SPM68 Projector x 2 (Reserved, flagged: the date or time changed); 4 in stock</t>
         </is>
       </c>
@@ -2003,7 +2076,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Short Kit' is in Planning, assigned to Daniel Tan, on 16 Sep 2027, 09:00-17:00. Its reservation of 2 SPM68 Speaker (Reserved) is flagged because Technical Support marked 1 of the 2 in stock out of service. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Short Kit' is in Planning, assigned to Daniel Tan, on 16 Oct 2027, 09:00-17:00. Its reservation of 2 SPM68 Speaker (Reserved) is flagged because Technical Support marked 1 of the 2 in stock out of service. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2103,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Short Kit (Planning), 16 Sep 2027, 09:00-17:00
+          <t>Event: SPM68 Short Kit (Planning), 16 Oct 2027, 09:00-17:00
 Equipment: SPM68 Speaker x 2 (Reserved, flagged); 2 in stock, 1 out of service</t>
         </is>
       </c>
@@ -2353,7 +2426,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Ready To Confirm' is in Planning, assigned to Daniel Tan, on 20 Sep 2027, 09:00-17:00. It has one approved venue booking at SPM68 Annex that is not flagged, no equipment, and registration enabled with a capacity of 30 and an opening and closing date. Its registrations (8 registered) are flagged because the date or time changed. Logged in as Daniel Tan.</t>
+          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Ready To Confirm' is in Planning, assigned to Daniel Tan, on 20 Oct 2027, 09:00-17:00. It has one approved venue booking at SPM68 Annex that is not flagged, no equipment, and registration enabled with a capacity of 30 and an opening and closing date. Its registrations (8 registered) are flagged because the date or time changed. Logged in as Daniel Tan.</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2456,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Ready To Confirm (Planning), 20 Sep 2027, 09:00-17:00
+          <t>Event: SPM68 Ready To Confirm (Planning), 20 Oct 2027, 09:00-17:00
 Venue booking: SPM68 Annex (Approved, not flagged)
 Registrations: 8 registered, 0 on the waiting list (flagged: the date or time changed)</t>
         </is>
@@ -2533,7 +2606,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Sep 2027, 09:00-17:00, for 150 people in Theatre layout, and requires 'Fixed ceiling projector' and 'Step-free access'. Its approved booking at SPM68 Hall (8 Sep 2027, 09:00-17:00, Theatre, seats 100) is flagged. SPM68 Spare Room seats 200 in Theatre layout, has both required features and is free that day. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Oct 2027, 09:00-17:00, for 150 people in Theatre layout, and requires 'Fixed ceiling projector' and 'Step-free access'. Its approved booking at SPM68 Hall (8 Oct 2027, 09:00-17:00, Theatre, seats 100) is flagged. SPM68 Spare Room seats 200 in Theatre layout, has both required features and is free that day. Logged in as Daniel Tan. Nothing is changed in this case.</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2632,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM68 Outgrown Room, 150 people, Theatre; requires Fixed ceiling projector and Step-free access
-Flagged booking: SPM68 Hall, 8 Sep 2027, 09:00-17:00, Theatre
+Flagged booking: SPM68 Hall, 8 Oct 2027, 09:00-17:00, Theatre
 Replacement candidate: SPM68 Spare Room (Theatre seats 200)</t>
         </is>
       </c>
@@ -2572,7 +2645,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The 'Find a venue' page opens, saying 'Filled in from the flagged booking at SPM68 Hall. Change any filter and search again.' 'From' reads 8 Sep 2027, 09:00 and 'To' reads 8 Sep 2027, 17:00. 'Expected attendance' reads 150. 'Room layout' reads 'Theatre'. 'Step-free access' is ticked under 'Accessibility requirements' and 'Fixed ceiling projector' is ticked under 'Required facilities'; nothing else is ticked. The results include 'SPM68 Spare Room (SPM68-SPR)' with a 'Request booking' button, and do not include SPM68 Hall.</t>
+          <t>Step 2: The 'Find a venue' page opens, saying 'Filled in from the flagged booking at SPM68 Hall. Change any filter and search again.' 'From' reads 8 Oct 2027, 09:00 and 'To' reads 8 Oct 2027, 17:00. 'Expected attendance' reads 150. 'Room layout' reads 'Theatre'. 'Step-free access' is ticked under 'Accessibility requirements' and 'Fixed ceiling projector' is ticked under 'Required facilities'; nothing else is ticked. The results include 'SPM68 Spare Room (SPM68-SPR)' with a 'Request booking' button, and do not include SPM68 Hall.</t>
         </is>
       </c>
     </row>
@@ -2693,11 +2766,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Requesting a replacement venue adds a pending request and leaves the flagged booking, the event's information and its status unchanged</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>Requesting a replacement venue adds a pending request and leaves the flagged booking on the event record, and the event's information and status unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2705,7 +2778,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Sep 2027, 09:00-17:00, for 150 people in Theatre layout. Its approved booking at SPM68 Hall is flagged. SPM68 Spare Room seats 200 in Theatre layout and is free that day. Logged in as Daniel Tan.</t>
+          <t>Run npm run fixtures:spm68 before this case. Go straight on to SPM-68-TC16, which needs the request this case makes, and reset after that one; to stop here instead, run npm run fixtures:spm68 again now. 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Oct 2027, 09:00-17:00, for 150 people in Theatre layout. Its approved booking at SPM68 Hall is flagged. SPM68 Spare Room seats 200 in Theatre layout and is free that day. Logged in as Daniel Tan.</t>
         </is>
       </c>
     </row>
@@ -2735,9 +2808,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Outgrown Room (Planning), 8 Sep 2027, 09:00-17:00, 150 people, Theatre
+          <t>Event: SPM68 Outgrown Room (Planning), 8 Oct 2027, 09:00-17:00, 150 people, Theatre
 Flagged booking: SPM68 Hall (Approved)
-Replacement: SPM68 Spare Room, 8 Sep 2027, 09:00-17:00</t>
+Replacement: SPM68 Spare Room, 8 Oct 2027, 09:00-17:00</t>
         </is>
       </c>
     </row>
@@ -2749,11 +2822,375 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The 'Request a venue booking' page opens for SPM68 Spare Room, with Date 8 Sep 2027, Start time 09:00 and End time 17:00 filled in.
+          <t>Step 3: The 'Request a venue booking' page opens for SPM68 Spare Room, with Date 8 Oct 2027, Start time 09:00 and End time 17:00 filled in.
 Step 4: The message 'Booking request sent to Venue Staff.' is shown.
-Step 5: Under 'Booking requests', SPM68 Spare Room is listed as 'Pending' and SPM68 Hall is still listed as 'Approved', both for 8 Sep 2027, 09:00–17:00.
-Step 6: The status badge still reads 'Planning'. The event still shows 8 Sep 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
+Step 5: Under 'Booking requests', SPM68 Spare Room is listed as 'Pending' and SPM68 Hall is still listed as 'Approved', both for 8 Oct 2027, 09:00–17:00.
+Step 6: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
 Step 7: The 'SPM68 Outgrown Room' item for SPM68 Hall is still listed under 'Venue bookings', still flagged, with 'Keep booking' and 'Find a replacement venue'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-68-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Releasing a flagged booking from the Flagged Arrangements page asks first, takes it off the page, keeps it on the event record as Released and leaves the replacement request and the event unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-68-TC15 has just been run ('SPM68 Outgrown Room' has a pending request for SPM68 Spare Room, and its flagged booking at SPM68 Hall is still Approved). Run npm run fixtures:spm68 after this case. Logged in as Daniel Tan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="139" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Flagged Arrangements' in the sidebar
+2. Click 'Release booking' in the 'SPM68 Outgrown Room' item
+3. Click 'Cancel' in the dialog
+4. Click 'Release booking' in the 'SPM68 Outgrown Room' item
+5. Type the reason in 'Reason (optional)'
+6. Click 'Release booking' in the dialog
+7. Click 'All Events' in the sidebar
+8. Click 'SPM68 Outgrown Room' in the list
+9. Click the 'Venue' tab
+10. Click the 'Readiness' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM68 Outgrown Room (Planning), 8 Oct 2027, 09:00-17:00, 150 people, Theatre
+Flagged booking: SPM68 Hall (Approved)
+Replacement request: SPM68 Spare Room (Pending)
+Reason: Room is too small for 150 people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="301" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: A dialog 'Release this booking?' reads 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 will be freed for other events, and Venue Staff will be notified.' It has an empty 'Reason (optional)' box and the buttons 'Release booking' and 'Cancel'.
+Step 3: The dialog closes. The 'SPM68 Outgrown Room' item is still listed and nothing was released.
+Step 6: The dialog closes. The message 'Booking released' is shown with 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 is now Released. Venue Staff have been notified.' The 'SPM68 Outgrown Room' item is no longer listed.
+Step 8: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
+Step 9: Under 'Booking requests', SPM68 Hall is still listed, now as 'Released' with 'Reason for release: Room is too small for 150 people.' and no button. SPM68 Spare Room is still 'Pending' for 8 Oct 2027, 09:00–17:00.
+Step 10: SPM68 Hall is not listed. 'SPM68 Spare Room' shows 'Pending' and 'Outstanding', and says it is still awaiting a decision from Venue Staff. The message '1 arrangement still blocks confirmation' is shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-68-TC17</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A flagged venue request that is still pending is withdrawn, not released, from the Flagged Arrangements page</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Pending Request' is in Planning, assigned to Daniel Tan, on 22 Oct 2027, 09:00-17:00, for 40 people in Theatre layout. Its only venue booking, a request for SPM68 Annex that Venue Staff have not decided (Pending), is flagged because the date or time changed. Logged in as Daniel Tan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Flagged Arrangements' in the sidebar
+2. Click 'Withdraw request' in the 'SPM68 Pending Request' item
+3. Click 'Withdraw request' in the dialog
+4. Click 'All Events' in the sidebar
+5. Click 'SPM68 Pending Request' in the list
+6. Click the 'Venue' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM68 Pending Request (Planning), 22 Oct 2027, 09:00-17:00, 40 people, Theatre
+Venue booking: SPM68 Annex (Pending, flagged: the date or time changed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: The 'SPM68 Pending Request' item shows 'SPM68 Annex (SPM68-ANX)' and 'Flagged because: the date or time changed', with the buttons 'Keep booking', 'Find a replacement venue' and 'Withdraw request'. It has no 'Release booking' button.
+Step 2: A dialog 'Withdraw this request?' reads 'SPM68 Annex (SPM68-ANX) on 22 Oct 2027, 09:00–17:00 will no longer be requested, and Venue Staff will no longer see it on their Booking Requests list.' It has an empty 'Reason (optional)' box and the buttons 'Withdraw request' and 'Cancel'.
+Step 3: The dialog closes. The message 'Request withdrawn' is shown with 'SPM68 Annex (SPM68-ANX) on 22 Oct 2027, 09:00–17:00 is now Withdrawn.' The 'SPM68 Pending Request' item is no longer listed.
+Step 6: Under 'Booking requests', SPM68 Annex is still listed, now as 'Withdrawn', with no reason line and no button.</t>
         </is>
       </c>
     </row>
@@ -2839,7 +3276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2875,13 +3312,13 @@
       </c>
       <c r="C2" s="11" t="n"/>
     </row>
-    <row r="3" ht="449.5" customHeight="1">
+    <row r="3" ht="463" customHeight="1">
       <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>The fixture script scripts/seed-spm68.ts (npm run fixtures:spm68) is NOT written yet, although the schema it needs exists. It is left to the build step because several fixture states only mean something once the live check is built (a booking that does not cover the event's time, a reservation left short), and it cannot be tried against the shared database blind. It needs, all titled 'SPM68 …' with seed keys 'spm68_…', organiser Rachel Ng, coordinator Daniel Tan unless said, status Planning: (1) dedicated venues, upserted as scripts/seed-spm81.ts does: SPM68 Hall (SPM68-HAL; Theatre 100, Classroom 60), SPM68 Annex (SPM68-ANX; Theatre 60), SPM68 Spare Room (SPM68-SPR; Theatre 200), SPM68 Closed Room (SPM68-CLS; Theatre 60; unavailable for maintenance 9 Sep 2027 08:00-18:00), SPM68 Retired Room (SPM68-RET; Theatre 60; retired) - all 07:00-22:00, no setup or turnaround, all with 'Fixed ceiling projector' and 'Step-free access'; (2) dedicated equipment: SPM68 Projector (4 in stock), SPM68 Speaker (2 in stock, 1 out of service); (3) events: Listing Summit (7 Sep 2027; Hall approved + flagged event_schedule_changed,event_requirements_changed; Annex approved, not flagged; Projector x 2 reserved + flagged event_schedule_changed; 12 registered + 3 waitlisted, flagged event_schedule_changed), Attendance Review (6 Sep; 80 people; Hall flagged event_attendance_changed), Outgrown Room (8 Sep; 150 people; requires both facilities; Hall flagged event_attendance_changed), Venue Trouble Day (9 Sep; Closed Room flagged venue_unavailable; Retired Room flagged venue_retired), Moved Date (event 14 Sep, Annex booking 13 Sep, flagged event_schedule_changed), Kit Recheck (15 Sep; Projector x 2 reserved, flagged event_schedule_changed), Short Kit (16 Sep; Speaker x 2 reserved, flagged equipment_unavailable), Capacity Cut (17 Sep; registration capacity 10; 12 registered + 3 waitlisted; flagged registration_capacity_lowered), Registration Off (18 Sep; registration off; 5 registered; flagged registration_disabled), Ready To Confirm (20 Sep; Annex approved, not flagged; registration capacity 30 with opening and closing dates; 8 registered; flagged event_schedule_changed), Partner Briefing (21 Sep; coordinator Priya Raj; Annex flagged event_attendance_changed). All times 09:00-17:00.</t>
+          <t>The fixture script scripts/seed-spm68.ts (npm run fixtures:spm68) is NOT written yet, although the schema it needs exists. It is left to the build step because several fixture states only mean something once the live check is built (a booking that does not cover the event's time, a reservation left short), and it cannot be tried against the shared database blind. It needs, all titled 'SPM68 …' with seed keys 'spm68_…', organiser Rachel Ng, coordinator Daniel Tan unless said, status Planning: (1) dedicated venues, upserted as scripts/seed-spm81.ts does: SPM68 Hall (SPM68-HAL; Theatre 100, Classroom 60), SPM68 Annex (SPM68-ANX; Theatre 60), SPM68 Spare Room (SPM68-SPR; Theatre 200), SPM68 Closed Room (SPM68-CLS; Theatre 60; unavailable for maintenance 9 Oct 2027 08:00-18:00), SPM68 Retired Room (SPM68-RET; Theatre 60; retired) - all 07:00-22:00, no setup or turnaround, all with 'Fixed ceiling projector' and 'Step-free access'; (2) dedicated equipment: SPM68 Projector (4 in stock), SPM68 Speaker (2 in stock, 1 out of service); (3) events: Listing Summit (7 Oct 2027; Hall approved + flagged event_schedule_changed,event_requirements_changed; Annex approved, not flagged; Projector x 2 reserved + flagged event_schedule_changed; 12 registered + 3 waitlisted, flagged event_schedule_changed), Attendance Review (6 Oct; 80 people; Hall flagged event_attendance_changed), Outgrown Room (8 Oct; 150 people; requires both facilities; Hall flagged event_attendance_changed), Venue Trouble Day (9 Oct; Closed Room flagged venue_unavailable; Retired Room flagged venue_retired), Moved Date (event 14 Oct, Annex booking 13 Oct, flagged event_schedule_changed), Kit Recheck (15 Oct; Projector x 2 reserved, flagged event_schedule_changed), Short Kit (16 Oct; Speaker x 2 reserved, flagged equipment_unavailable), Capacity Cut (17 Oct; registration capacity 10; 12 registered + 3 waitlisted; flagged registration_capacity_lowered), Registration Off (18 Oct; registration off; 5 registered; flagged registration_disabled), Ready To Confirm (20 Oct; Annex approved, not flagged; registration capacity 30 with opening and closing dates; 8 registered; flagged event_schedule_changed), Partner Briefing (21 Oct; coordinator Priya Raj; Annex flagged event_attendance_changed), Pending Request (22 Oct; 40 people; Annex PENDING, flagged event_schedule_changed). All times 09:00-17:00.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
@@ -3006,6 +3443,17 @@
         </is>
       </c>
       <c r="C14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="193" customHeight="1">
+      <c r="A15" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-13: releasing from the Flagged Arrangements page (AC12). A flagged booking's item has 'Release booking' when the booking is Approved and 'Withdraw request' when it is still Pending. Both use Withdraw or Release Venue Booking (SPM-67) exactly as the event's Venue tab does - the same question, optional reason, rules, notification to Venue Staff and refusals - so nothing new is built on the server. Two differences in wording: the dialog's other button is 'Cancel', not the Venue tab's 'Keep booking', because on this page 'Keep booking' is the button that clears the flag; and the message afterwards ends at 'Venue Staff have been notified.' ('… is now Withdrawn.' for a withdrawal), without 'You can request another venue below.' A withdrawn or released booking holds nothing, so it leaves the page and stops blocking confirmation; its flag is not separately cleared. The notification to Venue Staff is SPM-67's (SPM-67-TC03) and is not re-tested here.</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3065,7 +3513,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Listing Summit' is in Planning, assigned to Daniel Tan, on 7 Sep 2027, 09:00-17:00, for 50 people in Theatre layout. It has two approved venue bookings: SPM68 Hall (flagged for review) and SPM68 Annex (not flagged). Its reservation of 2 SPM68 Projector is flagged, and so are its registrations (12 registered, 3 on the waiting list). Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123). Nothing is changed in this case. Other stories' fixtures may add items to the same page; check only the items named here.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Listing Summit' is in Planning, assigned to Daniel Tan, on 7 Oct 2027, 09:00-17:00, for 50 people in Theatre layout. It has two approved venue bookings: SPM68 Hall (flagged for review) and SPM68 Annex (not flagged). Its reservation of 2 SPM68 Projector is flagged, and so are its registrations (12 registered, 3 on the waiting list). Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123). Nothing is changed in this case. Other stories' fixtures may add items to the same page; check only the items named here.</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3539,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Listing Summit (Planning), 7 Sep 2027, 09:00-17:00, 50 people, Theatre
+          <t>Event: SPM68 Listing Summit (Planning), 7 Oct 2027, 09:00-17:00, 50 people, Theatre
 Venue bookings: SPM68 Hall (Approved, flagged), SPM68 Annex (Approved, not flagged)
 Equipment: SPM68 Projector x 2 (Reserved, flagged); 4 in stock
 Registrations: 12 registered, 3 on the waiting list (flagged)
@@ -3107,7 +3555,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'Flagged Arrangements' page opens, with the link after 'Review Queue' in the sidebar. Under 'Venue bookings' there is an item for 'SPM68 Listing Summit' showing 'SPM68 Hall (SPM68-HAL)', '7 Sep 2027, 09:00–17:00', 'Theatre', 'Flagged because: the date or time changed; the venue requirements changed', 'Suitability: Suitable' and 'Availability: Available', with the buttons 'Keep booking' and 'Find a replacement venue'. There is no item for SPM68 Annex. Under 'Equipment reservations' there is an item for 'SPM68 Listing Summit' showing 'SPM68 Projector', 'Flagged because: the date or time changed' and 'Availability: 2 reserved, 4 available for these dates.', with the button 'Keep reservation'. Under 'Registrations' there is an item for 'SPM68 Listing Summit' showing '12 registered, 3 on the waiting list' and 'Flagged because: the date or time changed', with the button 'Mark as reviewed'.
+          <t>Step 1: The 'Flagged Arrangements' page opens, with the link after 'Review Queue' in the sidebar. Under 'Venue bookings' there is an item for 'SPM68 Listing Summit' showing 'SPM68 Hall (SPM68-HAL)', '7 Oct 2027, 09:00–17:00', 'Theatre', 'Flagged because: the date or time changed; the venue requirements changed', 'Suitability: Suitable' and 'Availability: Available', with the buttons 'Keep booking', 'Find a replacement venue' and 'Release booking'. There is no item for SPM68 Annex. Under 'Equipment reservations' there is an item for 'SPM68 Listing Summit' showing 'SPM68 Projector', 'Flagged because: the date or time changed' and 'Availability: 2 reserved, 4 available for these dates.', with the button 'Keep reservation'. Under 'Registrations' there is an item for 'SPM68 Listing Summit' showing '12 registered, 3 on the waiting list' and 'Flagged because: the date or time changed', with the button 'Mark as reviewed'.
 Step 2: The event's Overview opens, with the status badge 'Planning'.
 Step 3: Under 'Booking requests', both SPM68 Hall and SPM68 Annex are listed as 'Approved'.</t>
         </is>
@@ -3242,7 +3690,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Listing Summit' is assigned to Daniel Tan and has a flagged booking at SPM68 Hall. 'SPM68 Partner Briefing' is assigned to Priya Raj and has a flagged booking at SPM68 Annex on 21 Sep 2027. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Listing Summit' is assigned to Daniel Tan and has a flagged booking at SPM68 Hall. 'SPM68 Partner Briefing' is assigned to Priya Raj and has a flagged booking at SPM68 Annex on 21 Oct 2027. Logged in as Daniel Tan. Nothing is changed in this case.</t>
         </is>
       </c>
     </row>
@@ -3765,7 +4213,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Attendance Review' is in Planning, assigned to Daniel Tan, on 6 Sep 2027, 09:00-17:00, for 80 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. It has no equipment and registration is not enabled. Logged in as Daniel Tan. Confirmation is refused in this case, so nothing is changed.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Attendance Review' is in Planning, assigned to Daniel Tan, on 6 Oct 2027, 09:00-17:00, for 80 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. It has no equipment and registration is not enabled. Logged in as Daniel Tan. Confirmation is refused in this case, so nothing is changed.</t>
         </is>
       </c>
     </row>
@@ -3795,7 +4243,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Attendance Review (Planning), 6 Sep 2027, 09:00-17:00, 80 people, Theatre
+          <t>Event: SPM68 Attendance Review (Planning), 6 Oct 2027, 09:00-17:00, 80 people, Theatre
 Venue booking: SPM68 Hall (Approved, flagged: the expected attendance changed)</t>
         </is>
       </c>
@@ -3810,7 +4258,7 @@
         <is>
           <t>Step 3: 'SPM68 Hall' shows 'Approved' and 'Outstanding', and says it is flagged for review: the expected attendance changed. The message '1 arrangement still blocks confirmation' is shown.
 Step 6: The event is NOT confirmed. The message 'This event cannot be confirmed yet: SPM68 Hall for this event is flagged for review: the expected attendance changed.' is shown. The status badge still reads 'Planning'.
-Step 7: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 6 Sep 2027, 09:00–17:00. It was not changed or cancelled.</t>
+Step 7: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 6 Oct 2027, 09:00–17:00. It was not changed or cancelled.</t>
         </is>
       </c>
     </row>
@@ -3943,7 +4391,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Attendance Review' is in Planning, assigned to Daniel Tan, on 6 Sep 2027, 09:00-17:00, for 80 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. It has no equipment and registration is not enabled. Logged in as Daniel Tan.</t>
+          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Attendance Review' is in Planning, assigned to Daniel Tan, on 6 Oct 2027, 09:00-17:00, for 80 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. It has no equipment and registration is not enabled. Logged in as Daniel Tan.</t>
         </is>
       </c>
     </row>
@@ -3972,7 +4420,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Attendance Review (Planning), 6 Sep 2027, 09:00-17:00, 80 people, Theatre
+          <t>Event: SPM68 Attendance Review (Planning), 6 Oct 2027, 09:00-17:00, 80 people, Theatre
 Venue booking: SPM68 Hall (Approved, Theatre seats 100, flagged: the expected attendance changed)</t>
         </is>
       </c>
@@ -3987,7 +4435,7 @@
         <is>
           <t>Step 1: Under 'Venue bookings', the 'SPM68 Attendance Review' item shows 'SPM68 Hall (SPM68-HAL)', 'Flagged because: the expected attendance changed', 'Suitability: Suitable' and 'Availability: Available'.
 Step 2: The message 'Flag cleared' is shown with 'SPM68 Hall for SPM68 Attendance Review was kept as it is.' The 'SPM68 Attendance Review' item is no longer listed.
-Step 5: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 6 Sep 2027, 09:00–17:00 in Theatre layout. Its venue, times, layout and status are unchanged.
+Step 5: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 6 Oct 2027, 09:00–17:00 in Theatre layout. Its venue, times, layout and status are unchanged.
 Step 6: 'SPM68 Hall' shows 'Approved' and 'Complete', with no mention of being flagged. The message 'Nothing is blocking confirmation' is shown.</t>
         </is>
       </c>
@@ -4121,7 +4569,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Sep 2027, 09:00-17:00, for 150 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Oct 2027, 09:00-17:00, for 150 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4597,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM68 Outgrown Room (Planning), 8 Sep 2027, 09:00-17:00, 150 people, Theatre
+          <t>Event: SPM68 Outgrown Room (Planning), 8 Oct 2027, 09:00-17:00, 150 people, Theatre
 Venue booking: SPM68 Hall (Approved, Theatre seats 100, flagged: the expected attendance changed)</t>
         </is>
       </c>
@@ -4165,7 +4613,7 @@
           <t>Step 1: The 'SPM68 Outgrown Room' item shows 'Flagged because: the expected attendance changed', 'Suitability: Not suitable' with 'Theatre capacity is 100 - your event expects 150.', and 'Availability: Available'.
 Step 2: The flag is NOT cleared. The message 'SPM68 Hall no longer meets this event's requirements: Theatre capacity is 100 - your event expects 150.' is shown in the item. The item is still listed, with 'Keep booking' and 'Find a replacement venue'.
 Step 3: The 'SPM68 Outgrown Room' item is still listed with 'Suitability: Not suitable'.
-Step 5: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Sep 2027, 09:00–17:00. It was not changed or cancelled.</t>
+Step 5: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Oct 2027, 09:00–17:00. It was not changed or cancelled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-68: the flagged page only clears flags; Keep only when it still fits
- Release booking and Withdraw request are off the Flagged Arrangements
  page. Each flagged booking links to its event's Venue tab, where
  SPM-67 already does both. AC12 asks only that the flagged booking stays
  until it is released.
- Keep booking and Keep reservation are offered only while the
  arrangement still meets the event's requirements. Otherwise the item
  lists what is unmet and says it can't be kept. The server still
  refuses, for a page showing an older result.
- Equipment items link to the event's Equipment tab, and registrations
  items to its Overview, where the registration settings are changed.
- Manual cases 15 -> 14: the withdraw-from-the-page case and its fixture
  event are removed; the refused-keep cases check that Keep is absent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-68_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-68_Test_Cases.xlsx
@@ -22,7 +22,6 @@
     <sheet name="TC12" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -462,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -694,7 +693,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>A flagged venue booking whose room is now too small cannot be kept: the flag stays and the unmet requirement is named</t>
+          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking': the unmet requirement is named, the flag stays and the booking is unchanged</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -726,7 +725,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Flagged bookings at a blocked venue and at a retired venue are shown as not available with the reason, and neither can be kept</t>
+          <t>Flagged bookings at a blocked venue and at a retired venue are shown as not available with the reason, and neither is offered 'Keep booking'</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -758,7 +757,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>A flagged venue booking that no longer covers the event's new date is shown as not available and cannot be kept</t>
+          <t>A flagged venue booking that no longer covers the event's new date is shown as not available and is not offered 'Keep booking'</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -822,7 +821,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>A flagged equipment reservation that can no longer be covered cannot be kept: the flag stays and the shortfall is named</t>
+          <t>A flagged equipment reservation that can no longer be covered is not offered 'Keep reservation': the shortfall is named, the flag stays and the reservation is unchanged</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -854,7 +853,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Flagged registrations show how many attendees are registered or waitlisted and why, and marking them as reviewed clears the flag without changing the registration settings</t>
+          <t>Flagged registrations show how many attendees are registered or waitlisted and why, link to the event's Overview where the registration settings are changed, and marking them as reviewed clears the flag without changing those settings</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -950,7 +949,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Releasing a flagged booking from the Flagged Arrangements page asks first, takes it off the page, keeps it on the event record as Released and leaves the replacement request and the event unchanged</t>
+          <t>The flagged booking is released from the event's Venue tab, reached from the Flagged Arrangements page; it then leaves the page, stays on the event record as Released, and the replacement request and the event are unchanged</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -969,72 +968,40 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>TC15</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC15</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>A flagged venue request that is still pending is withdrawn, not released, from the Flagged Arrangements page</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>AC12, AC14</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Boundary</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
         </is>
       </c>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="9" t="n"/>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC02
@@ -1042,22 +1009,22 @@
 SPM-68-TC04</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Each flagged arrangement shows the event, the arrangement, and why it was flagged (e.g. event date changed, attendance changed, venue attributes updated, venue setup or turnaround time changed, venue retired, venue blocked, equipment marked unavailable).</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC07
@@ -1065,42 +1032,42 @@
 SPM-68-TC10</t>
         </is>
       </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="31" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Given an event has more than one venue booking, when one of them is flagged, then only the flagged booking is listed.</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC01</t>
+        </is>
+      </c>
       <c r="F23" s="9" t="n"/>
     </row>
-    <row r="24" ht="31" customHeight="1">
+    <row r="24" ht="71.5" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Given an event has more than one venue booking, when one of them is flagged, then only the flagged booking is listed.</t>
+          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="71.5" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC05
@@ -1109,65 +1076,65 @@
 SPM-68-TC08</t>
         </is>
       </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="44.5" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>For a flagged equipment reservation, the current availability result for the event's present dates and quantities is shown.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC01
+SPM-68-TC09
+SPM-68-TC10</t>
+        </is>
+      </c>
       <c r="F25" s="9" t="n"/>
     </row>
     <row r="26" ht="44.5" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>For a flagged equipment reservation, the current availability result for the event's present dates and quantities is shown.</t>
+          <t>Given the arrangement still meets the event's requirements, when the Coordinator keeps it, then the flag is cleared and the arrangement is unchanged.</t>
         </is>
       </c>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC01
-SPM-68-TC09
-SPM-68-TC10</t>
+          <t>SPM-68-TC05
+SPM-68-TC09</t>
         </is>
       </c>
       <c r="F26" s="9" t="n"/>
     </row>
-    <row r="27" ht="44.5" customHeight="1">
+    <row r="27" ht="58" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Given the arrangement still meets the event's requirements, when the Coordinator keeps it, then the flag is cleared and the arrangement is unchanged.</t>
+          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC05
-SPM-68-TC09</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC06
 SPM-68-TC07
@@ -1175,98 +1142,119 @@
 SPM-68-TC10</t>
         </is>
       </c>
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="71.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>AC8</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>For flagged registrations, the number of attendees registered or on the waiting list is shown, with why they were flagged: the event's date or time changed (see: Update Event Information, SPM-62), or the registration capacity was lowered below the number registered or registration was turned off (see: Configure Event Registration, SPM-64).</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC01
+SPM-68-TC11</t>
+        </is>
+      </c>
       <c r="F28" s="9" t="n"/>
     </row>
-    <row r="29" ht="71.5" customHeight="1">
+    <row r="29" ht="31" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>AC8</t>
+          <t>AC9</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>For flagged registrations, the number of attendees registered or on the waiting list is shown, with why they were flagged: the event's date or time changed (see: Update Event Information, SPM-62), or the registration capacity was lowered below the number registered or registration was turned off (see: Configure Event Registration, SPM-64).</t>
+          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC01
-SPM-68-TC11</t>
+          <t>SPM-68-TC11</t>
         </is>
       </c>
       <c r="F29" s="9" t="n"/>
     </row>
-    <row r="30" ht="31" customHeight="1">
+    <row r="30" ht="17.5" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>AC9</t>
+          <t>AC10</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
+          <t>Flagged registrations do not prevent confirmation.</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC11</t>
+          <t>SPM-68-TC12</t>
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
     </row>
-    <row r="31" ht="17.5" customHeight="1">
+    <row r="31" ht="58" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>AC10</t>
+          <t>AC11</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Flagged registrations do not prevent confirmation.</t>
+          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC12</t>
+          <t>SPM-68-TC13</t>
         </is>
       </c>
       <c r="F31" s="9" t="n"/>
     </row>
-    <row r="32" ht="58" customHeight="1">
+    <row r="32" ht="44.5" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC12</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
+          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13</t>
+          <t>SPM-68-TC13
+SPM-68-TC14</t>
         </is>
       </c>
       <c r="F32" s="9" t="n"/>
     </row>
-    <row r="33" ht="44.5" customHeight="1">
+    <row r="33" ht="31" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC13</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
+          <t>Replacing a venue does not change the event's own information or status.</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
@@ -1274,47 +1262,25 @@
       <c r="E33" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC13
-SPM-68-TC14
-SPM-68-TC15</t>
+SPM-68-TC14</t>
         </is>
       </c>
       <c r="F33" s="9" t="n"/>
     </row>
-    <row r="34" ht="31" customHeight="1">
+    <row r="34" ht="98.5" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC14</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Replacing a venue does not change the event's own information or status.</t>
+          <t>A flagged arrangement is never changed or cancelled automatically.</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC13
-SPM-68-TC14</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n"/>
-    </row>
-    <row r="35" ht="112" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>AC14</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>A flagged arrangement is never changed or cancelled automatically.</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC05
 SPM-68-TC06
@@ -1322,59 +1288,58 @@
 SPM-68-TC09
 SPM-68-TC10
 SPM-68-TC13
-SPM-68-TC14
-SPM-68-TC15</t>
+SPM-68-TC14</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="44.5" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>AC15</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>A flagged venue booking or equipment reservation counts as outstanding and prevents confirmation until it is resolved (see: Track Outstanding Arrangements).</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC05</t>
         </is>
       </c>
       <c r="F35" s="9" t="n"/>
     </row>
-    <row r="36" ht="44.5" customHeight="1">
+    <row r="36" ht="31" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>AC15</t>
+          <t>AC16</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>A flagged venue booking or equipment reservation counts as outstanding and prevents confirmation until it is resolved (see: Track Outstanding Arrangements).</t>
+          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
         </is>
       </c>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC05</t>
+          <t>SPM-68-TC02</t>
         </is>
       </c>
       <c r="F36" s="9" t="n"/>
     </row>
-    <row r="37" ht="31" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>AC16</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC02</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n"/>
-    </row>
-    <row r="39" ht="274" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="38" ht="260.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>prisma/schema.prisma
 prisma/seed.ts
@@ -1392,16 +1357,15 @@
 src/lib/flaggedArrangementsService.ts
 src/lib/roles.ts
 src/lib/validation/events.ts
-src/lib/venueBookingChange.ts
 src/lib/venueConflict.ts
 src/lib/venueSearchForm.ts
 src/lib/venueSuitability.ts</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="9" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="36">
@@ -1413,18 +1377,19 @@
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E35:F35"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E20:F20"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="E31:F31"/>
+    <mergeCell ref="B20:D20"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="E30:F30"/>
+    <mergeCell ref="B38:F38"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B26:D26"/>
@@ -1437,7 +1402,6 @@
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E37:F37"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E21:F21"/>
@@ -1457,7 +1421,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1496,7 +1459,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1504,7 +1467,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A flagged venue booking that no longer covers the event's new date is shown as not available and cannot be kept</t>
+          <t>A flagged venue booking that no longer covers the event's new date is shown as not available and is not offered 'Keep booking'</t>
         </is>
       </c>
     </row>
@@ -1516,11 +1479,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Moved Date' is in Planning, assigned to Daniel Tan, for 40 people in Theatre layout. The event was moved to 14 Oct 2027, 09:00-17:00, but its approved booking at SPM68 Annex is still for 13 Oct 2027, 09:00-17:00 and is flagged because the date or time changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Moved Date' is in Planning, assigned to Daniel Tan, for 40 people in Theatre layout. The event was moved to 14 Oct 2027, 09:00-17:00, but its approved booking at SPM68 Annex is still for 13 Oct 2027, 09:00-17:00 and is flagged because the date or time changed. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1528,8 +1491,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Flagged Arrangements' in the sidebar
-2. Click 'Keep booking' in the 'SPM68 Moved Date' item</t>
+          <t>1. Click 'Flagged Arrangements' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1508,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="152.5" customHeight="1">
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1554,8 +1516,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'SPM68 Moved Date' item shows 'SPM68 Annex (SPM68-ANX)', '13 Oct 2027, 09:00–17:00', 'Flagged because: the date or time changed', 'Suitability: Suitable' and 'Availability: Not available' with 'The booking (13 Oct 2027, 09:00–17:00) does not cover the event's time (14 Oct 2027, 09:00–17:00).'
-Step 2: The flag is NOT cleared. The message 'SPM68 Annex no longer meets this event's requirements: The booking (13 Oct 2027, 09:00–17:00) does not cover the event's time (14 Oct 2027, 09:00–17:00).' is shown in the item, and the item is still listed with the booking still on 13 Oct 2027.</t>
+          <t>Step 1: The 'SPM68 Moved Date' item shows 'SPM68 Annex (SPM68-ANX)', '13 Oct 2027, 09:00–17:00', 'Flagged because: the date or time changed', 'Suitability: Suitable' and 'Availability: Not available' with 'The booking (13 Oct 2027, 09:00–17:00) does not cover the event's time (14 Oct 2027, 09:00–17:00).' It shows 'This booking can't be kept while it doesn't meet the event's requirements.' and has no 'Keep booking' button.</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1806,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1853,7 +1814,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A flagged equipment reservation that can no longer be covered cannot be kept: the flag stays and the shortfall is named</t>
+          <t>A flagged equipment reservation that can no longer be covered is not offered 'Keep reservation': the shortfall is named, the flag stays and the reservation is unchanged</t>
         </is>
       </c>
     </row>
@@ -1865,11 +1826,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Short Kit' is in Planning, assigned to Daniel Tan, on 16 Oct 2027, 09:00-17:00. Its reservation of 2 SPM68 Speaker (Reserved) is flagged because Technical Support marked 1 of the 2 in stock out of service. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="71.5" customHeight="1">
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Short Kit' is in Planning, assigned to Daniel Tan, on 16 Oct 2027, 09:00-17:00. Its reservation of 2 SPM68 Speaker (Reserved) is flagged because Technical Support marked 1 of the 2 in stock out of service. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1879,9 +1840,7 @@
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
 2. Click the 'Equipment reservations' tab
-3. Click 'Keep reservation' in the 'SPM68 Short Kit' item
-4. Click 'SPM68 Short Kit' in its item
-5. Click the 'Equipment' tab</t>
+3. Click 'Open Equipment tab' in the 'SPM68 Short Kit' item</t>
         </is>
       </c>
     </row>
@@ -1906,9 +1865,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: On the 'Equipment reservations' tab, the 'SPM68 Short Kit' item shows 'SPM68 Speaker', 'Flagged because: units of the equipment were marked out of service' and 'Availability: 2 reserved, 1 available for these dates.'
-Step 3: The flag is NOT cleared. The message 'SPM68 Speaker no longer meets this event's requirements: 2 reserved, 1 available for these dates.' is shown in the item, and the item is still listed.
-Step 5: SPM68 Speaker is still listed with quantity 2 and the status 'Reserved'. It was not changed or cancelled.</t>
+          <t>Step 2: On the 'Equipment reservations' tab, the 'SPM68 Short Kit' item shows 'SPM68 Speaker', 'Flagged because: units of the equipment were marked out of service', 'Availability: 2 reserved, 1 available for these dates.' and 'This reservation can't be kept while it doesn't meet the event's requirements.' It has no 'Keep reservation' button. It has 'Open Equipment tab'.
+Step 3: The event's Equipment tab opens. SPM68 Speaker is still listed with quantity 2 and the status 'Reserved'. It was not changed or cancelled.</t>
         </is>
       </c>
     </row>
@@ -2021,7 +1979,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -2029,7 +1987,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Flagged registrations show how many attendees are registered or waitlisted and why, and marking them as reviewed clears the flag without changing the registration settings</t>
+          <t>Flagged registrations show how many attendees are registered or waitlisted and why, link to the event's Overview where the registration settings are changed, and marking them as reviewed clears the flag without changing those settings</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2003,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="71.5" customHeight="1">
+    <row r="5" ht="125.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2055,9 +2013,12 @@
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
 2. Click the 'Registrations' tab
-3. Click 'Mark as reviewed' in the 'SPM68 Capacity Cut' item
-4. Click 'All Events' in the sidebar
-5. Click 'SPM68 Capacity Cut' in the list</t>
+3. Click 'Open Overview' in the 'SPM68 Registration Off' item
+4. Click 'Flagged Arrangements' in the sidebar
+5. Click the 'Registrations' tab
+6. Click 'Mark as reviewed' in the 'SPM68 Capacity Cut' item
+7. Click 'All Events' in the sidebar
+8. Click 'SPM68 Capacity Cut' in the list</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="206.5" customHeight="1">
+    <row r="7" ht="260.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2082,9 +2043,10 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: On the 'Registrations' tab, the 'SPM68 Capacity Cut' item shows '12 registered, 3 on the waiting list' and 'Flagged because: the registration capacity was lowered below the number registered or waitlisted'. The 'SPM68 Registration Off' item shows '5 registered, 0 on the waiting list' and 'Flagged because: registration was turned off'. Each has a 'Mark as reviewed' button and no 'Keep' button.
-Step 3: The message 'Flag cleared' is shown with 'Registrations for SPM68 Capacity Cut were marked as reviewed. No registration was changed.' The 'SPM68 Capacity Cut' item is no longer listed. The 'SPM68 Registration Off' item is still listed.
-Step 5: On the Overview, the Registration card still shows Registration 'Enabled' and Capacity '10'. The status badge still reads 'Planning'.</t>
+          <t>Step 2: On the 'Registrations' tab, the 'SPM68 Capacity Cut' item shows '12 registered, 3 on the waiting list' and 'Flagged because: the registration capacity was lowered below the number registered or waitlisted'. The 'SPM68 Registration Off' item shows '5 registered, 0 on the waiting list' and 'Flagged because: registration was turned off'. Each has the buttons 'Mark as reviewed' and 'Open Overview', and no 'Keep' button.
+Step 3: The Overview of 'SPM68 Registration Off' opens. Its Registration card shows Registration 'Not enabled for this event' and has a 'Change registration settings' button.
+Step 6: The message 'Flag cleared' is shown with 'Registrations for SPM68 Capacity Cut were marked as reviewed. No registration was changed.' The 'SPM68 Capacity Cut' item is no longer listed. The 'SPM68 Registration Off' item is still listed.
+Step 8: On the Overview, the Registration card still shows Registration 'Enabled' and Capacity '10'. The status badge still reads 'Planning'.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2397,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="314.5" customHeight="1">
+    <row r="7" ht="328" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2448,7 +2410,7 @@
 Step 4: The message 'Booking request sent to Venue Staff.' is shown.
 Step 5: Under 'Booking requests', SPM68 Spare Room is listed as 'Pending' and SPM68 Hall is still listed as 'Approved', both for 8 Oct 2027, 09:00–17:00.
 Step 6: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
-Step 7: The 'SPM68 Outgrown Room' item for SPM68 Hall is still listed on the 'Venue bookings' tab, still flagged, with 'Keep booking' and 'Find a replacement venue'.</t>
+Step 7: The 'SPM68 Outgrown Room' item for SPM68 Hall is still listed on the 'Venue bookings' tab, still flagged, with 'Keep booking', 'Find a replacement venue' and 'Open Venue tab'.</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2531,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Releasing a flagged booking from the Flagged Arrangements page asks first, takes it off the page, keeps it on the event record as Released and leaves the replacement request and the event unchanged</t>
+          <t>The flagged booking is released from the event's Venue tab, reached from the Flagged Arrangements page; it then leaves the page, stays on the event record as Released, and the replacement request and the event are unchanged</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2547,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="139" customHeight="1">
+    <row r="5" ht="125.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2594,15 +2556,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
-2. Click 'Release booking' in the 'SPM68 Outgrown Room' item
-3. Click 'Cancel' in the dialog
-4. Click 'Release booking' in the 'SPM68 Outgrown Room' item
-5. Type the reason in 'Reason (optional)'
-6. Click 'Release booking' in the dialog
-7. Click 'All Events' in the sidebar
-8. Click 'SPM68 Outgrown Room' in the list
-9. Click the 'Venue' tab
-10. Click the 'Readiness' tab</t>
+2. Click 'Open Venue tab' in the 'SPM68 Outgrown Room' item
+3. Click 'Release booking' on the 'SPM68 Hall (SPM68-HAL)' row of the 'Booking requests' card
+4. Type the reason in 'Reason (optional)'
+5. Click 'Release booking' in the dialog
+6. Click the 'Overview' tab
+7. Click the 'Readiness' tab
+8. Click 'Flagged Arrangements' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2581,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="301" customHeight="1">
+    <row r="7" ht="328" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2629,190 +2589,13 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: A dialog 'Release this booking?' reads 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 will be freed for other events, and Venue Staff will be notified.' It has an empty 'Reason (optional)' box and the buttons 'Release booking' and 'Cancel'.
-Step 3: The dialog closes. The 'SPM68 Outgrown Room' item is still listed and nothing was released.
-Step 6: The dialog closes. The message 'Booking released' is shown with 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 is now Released. Venue Staff have been notified.' The 'SPM68 Outgrown Room' item is no longer listed.
-Step 8: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
-Step 9: Under 'Booking requests', SPM68 Hall is still listed, now as 'Released' with 'Reason for release: Room is too small for 150 people.' and no button. SPM68 Spare Room is still 'Pending' for 8 Oct 2027, 09:00–17:00.
-Step 10: SPM68 Hall is not listed. 'SPM68 Spare Room' shows 'Pending' and 'Outstanding', and says it is still awaiting a decision from Venue Staff. The message '1 arrangement still blocks confirmation' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>kchoongg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>46308</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-68-TC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>A flagged venue request that is still pending is withdrawn, not released, from the Flagged Arrangements page</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Pending Request' is in Planning, assigned to Daniel Tan, on 22 Oct 2027, 09:00-17:00, for 40 people in Theatre layout. Its only venue booking, a request for SPM68 Annex that Venue Staff have not decided (Pending), is flagged because the date or time changed. Logged in as Daniel Tan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="98.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1. Click 'Flagged Arrangements' in the sidebar
-2. Click 'Withdraw request' in the 'SPM68 Pending Request' item
-3. Click 'Withdraw request' in the dialog
-4. Click 'All Events' in the sidebar
-5. Click 'SPM68 Pending Request' in the list
-6. Click the 'Venue' tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Event: SPM68 Pending Request (Planning), 22 Oct 2027, 09:00-17:00, 40 people, Theatre
-Venue booking: SPM68 Annex (Pending, flagged: the date or time changed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="220" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Step 1: The 'SPM68 Pending Request' item shows 'SPM68 Annex (SPM68-ANX)' and 'Flagged because: the date or time changed', with the buttons 'Keep booking', 'Find a replacement venue' and 'Withdraw request'. It has no 'Release booking' button.
-Step 2: A dialog 'Withdraw this request?' reads 'SPM68 Annex (SPM68-ANX) on 22 Oct 2027, 09:00–17:00 will no longer be requested, and Venue Staff will no longer see it on their Booking Requests list.' It has an empty 'Reason (optional)' box and the buttons 'Withdraw request' and 'Cancel'.
-Step 3: The dialog closes. The message 'Request withdrawn' is shown with 'SPM68 Annex (SPM68-ANX) on 22 Oct 2027, 09:00–17:00 is now Withdrawn.' The 'SPM68 Pending Request' item is no longer listed.
-Step 6: Under 'Booking requests', SPM68 Annex is still listed, now as 'Withdrawn', with no reason line and no button.</t>
+          <t>Step 1: The 'SPM68 Outgrown Room' item for SPM68 Hall is listed with 'Keep booking', 'Find a replacement venue' and 'Open Venue tab'. It has no 'Release booking' or 'Withdraw request' button.
+Step 2: The event's Venue tab opens. Under 'Booking requests', SPM68 Hall is 'Approved' with a 'Release booking' button and SPM68 Spare Room is 'Pending'.
+Step 3: A dialog 'Release this booking?' reads 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 will be freed for other events, and Venue Staff will be notified.'
+Step 5: The dialog closes. The message 'Booking released' is shown. SPM68 Hall is still listed, now as 'Released' with 'Reason for release: Room is too small for 150 people.' and no button. SPM68 Spare Room is still 'Pending' for 8 Oct 2027, 09:00–17:00.
+Step 6: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
+Step 7: SPM68 Hall is not listed. 'SPM68 Spare Room' shows 'Pending' and 'Outstanding', and says it is still awaiting a decision from Venue Staff. The message '1 arrangement still blocks confirmation' is shown.
+Step 8: On the 'Venue bookings' tab there is no longer an item for 'SPM68 Outgrown Room'.</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3011,13 +2794,13 @@
       </c>
       <c r="C9" s="11" t="n"/>
     </row>
-    <row r="10" ht="152.5" customHeight="1">
+    <row r="10" ht="166" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-13: the messages. Kept: 'Flag cleared' with '&lt;arrangement&gt; for &lt;event&gt; was kept as it is.' Registrations reviewed: 'Flag cleared' with 'Registrations for &lt;event&gt; were marked as reviewed. No registration was changed.' Refused: '&lt;arrangement&gt; no longer meets this event's requirements: &lt;each unmet requirement&gt;', shown inside the item, which stays listed. The unmet venue requirements use the existing wording ('Theatre capacity is 100 - your event expects 150.', '&lt;Venue&gt; is unavailable at this time (maintenance, …).') plus two new ones: '&lt;Venue&gt; has been retired.' and 'The booking (&lt;its times&gt;) does not cover the event's time (&lt;the event's times&gt;).' Keeping asks for no confirmation: it changes nothing but the flag.</t>
+          <t>DECIDED 2026-10-13: the messages. Kept: 'Flag cleared' with '&lt;arrangement&gt; for &lt;event&gt; was kept as it is.' Registrations reviewed: 'Flag cleared' with 'Registrations for &lt;event&gt; were marked as reviewed. No registration was changed.' Refused by the server: '&lt;arrangement&gt; no longer meets this event's requirements: &lt;each unmet requirement&gt;', shown inside the item, which stays listed - seen only when the page's result was out of date (see the decision on not offering Keep). The unmet venue requirements use the existing wording ('Theatre capacity is 100 - your event expects 150.', '&lt;Venue&gt; is unavailable at this time (maintenance, …).') plus two new ones: '&lt;Venue&gt; has been retired.' and 'The booking (&lt;its times&gt;) does not cover the event's time (&lt;the event's times&gt;).' Keeping asks for no confirmation: it changes nothing but the flag.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
@@ -3044,13 +2827,13 @@
       </c>
       <c r="C12" s="11" t="n"/>
     </row>
-    <row r="13" ht="193" customHeight="1">
+    <row r="13" ht="139" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-13: releasing from the Flagged Arrangements page (AC12). A flagged booking's item has 'Release booking' when the booking is Approved and 'Withdraw request' when it is still Pending. Both use Withdraw or Release Venue Booking (SPM-67) exactly as the event's Venue tab does - the same question, optional reason, rules, notification to Venue Staff and refusals - so nothing new is built on the server. Two differences in wording: the dialog's other button is 'Cancel', not the Venue tab's 'Keep booking', because on this page 'Keep booking' is the button that clears the flag; and the message afterwards ends at 'Venue Staff have been notified.' ('… is now Withdrawn.' for a withdrawal), without 'You can request another venue below.' A withdrawn or released booking holds nothing, so it leaves the page and stops blocking confirmation; its flag is not separately cleared. The notification to Venue Staff is SPM-67's (SPM-67-TC03) and is not re-tested here.</t>
+          <t>DECIDED 2026-10-13 (Kristen), replacing the decision of 2026-10-13: the Flagged Arrangements page has no 'Release booking' or 'Withdraw request' button. AC12 asks only that the flagged booking stays on the event record until the Coordinator releases it; releasing is Withdraw or Release Venue Booking (SPM-67), which is on the event's Venue tab, and a change to an event's bookings is made in that one place. The page clears flags and never changes an arrangement. Each flagged booking has an 'Open Venue tab' link to its event's Venue tab instead. A withdrawn or released booking holds nothing, so it leaves the page and stops blocking confirmation; its flag is not separately cleared (SPM-68-TC14).</t>
         </is>
       </c>
       <c r="C13" s="11" t="n"/>
@@ -3065,6 +2848,28 @@
         </is>
       </c>
       <c r="C14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="206.5" customHeight="1">
+      <c r="A15" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-13 (Kristen), changing how AC7 is met: 'Keep booking' and 'Keep reservation' are offered only while the arrangement still meets the event's requirements. Where it does not, the item lists what is unmet, says 'This booking can't be kept while it doesn't meet the event's requirements.' ('This reservation …' for equipment) and has no Keep button - offering to keep a booking the page itself shows as clashing made no sense. AC7 is worded as 'when the Coordinator attempts to keep it': its outcome still holds (the flag is not cleared and the unmet requirement is identified), but the attempt cannot be made from the screen, so SPM-68-TC06, SPM-68-TC07, SPM-68-TC08 and SPM-68-TC10 check that Keep is absent rather than clicking it. The server still refuses a keep of an arrangement that no longer fits, for a page showing an older result; that refusal is covered by the automated tests only. Every equipment item also has 'Open Equipment tab', so one that cannot be kept is not a dead end.</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="98.5" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-13 (Kristen): a registrations item also has 'Open Overview', a link to the event's Overview, where the Registration card's 'Change registration settings' (SPM-64) raises the capacity or turns registration back on. Like 'Open Venue tab' and 'Open Equipment tab', it only takes the Coordinator to where the change is made; the Flagged Arrangements page itself still changes nothing but the flag (SPM-68-TC01, SPM-68-TC11).</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3161,7 +2966,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="368.5" customHeight="1">
+    <row r="7" ht="382" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3169,9 +2974,9 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'Flagged Arrangements' page opens, with the link after 'Review Queue' in the sidebar. It has three tabs, 'Venue bookings', 'Equipment reservations' and 'Registrations', each followed by how many are flagged, and opens on 'Venue bookings'. There is an item for 'SPM68 Listing Summit' showing 'SPM68 Hall (SPM68-HAL)', '7 Oct 2027, 09:00–17:00', 'Theatre', 'Flagged because: the date or time changed; the venue requirements changed', 'Suitability: Suitable' and 'Availability: Available', with the buttons 'Keep booking', 'Find a replacement venue' and 'Release booking'. There is no item for SPM68 Annex. No equipment or registrations are shown on this tab.
-Step 2: The 'Equipment reservations' tab shows an item for 'SPM68 Listing Summit' with 'SPM68 Projector', 'Flagged because: the date or time changed' and 'Availability: 2 reserved, 4 available for these dates.', with the button 'Keep reservation'. No venue booking is shown on this tab.
-Step 3: The 'Registrations' tab shows an item for 'SPM68 Listing Summit' with '12 registered, 3 on the waiting list' and 'Flagged because: the date or time changed', with the button 'Mark as reviewed'.
+          <t>Step 1: The 'Flagged Arrangements' page opens, with the link after 'Review Queue' in the sidebar. It has three tabs, 'Venue bookings', 'Equipment reservations' and 'Registrations', each followed by how many are flagged, and opens on 'Venue bookings'. There is an item for 'SPM68 Listing Summit' showing 'SPM68 Hall (SPM68-HAL)', '7 Oct 2027, 09:00–17:00', 'Theatre', 'Flagged because: the date or time changed; the venue requirements changed', 'Suitability: Suitable' and 'Availability: Available', with the buttons 'Keep booking', 'Find a replacement venue' and 'Open Venue tab'. There is no item for SPM68 Annex. No equipment or registrations are shown on this tab.
+Step 2: The 'Equipment reservations' tab shows an item for 'SPM68 Listing Summit' with 'SPM68 Projector', 'Flagged because: the date or time changed' and 'Availability: 2 reserved, 4 available for these dates.', with the buttons 'Keep reservation' and 'Open Equipment tab'. No venue booking is shown on this tab.
+Step 3: The 'Registrations' tab shows an item for 'SPM68 Listing Summit' with '12 registered, 3 on the waiting list' and 'Flagged because: the date or time changed', with the buttons 'Mark as reviewed' and 'Open Overview'.
 Step 4: The 'SPM68 Listing Summit' item for SPM68 Hall is shown again.
 Step 5: The event's Overview opens, with the status badge 'Planning'.
 Step 6: Under 'Booking requests', both SPM68 Hall and SPM68 Annex are listed as 'Approved'.</t>
@@ -3996,7 +3801,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -4004,11 +3809,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A flagged venue booking whose room is now too small cannot be kept: the flag stays and the unmet requirement is named</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking': the unmet requirement is named, the flag stays and the booking is unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4016,11 +3821,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Oct 2027, 09:00-17:00, for 150 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="71.5" customHeight="1">
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Outgrown Room' is in Planning, assigned to Daniel Tan, on 8 Oct 2027, 09:00-17:00, for 150 people in Theatre layout. Its only venue booking, SPM68 Hall (Approved, Theatre seats 100), is flagged because the expected attendance changed. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4029,10 +3834,8 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
-2. Click 'Keep booking' in the 'SPM68 Outgrown Room' item
-3. Refresh the page in the browser
-4. Click 'SPM68 Outgrown Room' in its item
-5. Click the 'Venue' tab</t>
+2. Refresh the page in the browser
+3. Click 'Open Venue tab' in the 'SPM68 Outgrown Room' item</t>
         </is>
       </c>
     </row>
@@ -4049,7 +3852,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="193" customHeight="1">
+    <row r="7" ht="179.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4057,10 +3860,9 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'SPM68 Outgrown Room' item shows 'Flagged because: the expected attendance changed', 'Suitability: Not suitable' with 'Theatre capacity is 100 - your event expects 150.', and 'Availability: Available'.
-Step 2: The flag is NOT cleared. The message 'SPM68 Hall no longer meets this event's requirements: Theatre capacity is 100 - your event expects 150.' is shown in the item. The item is still listed, with 'Keep booking' and 'Find a replacement venue'.
-Step 3: The 'SPM68 Outgrown Room' item is still listed with 'Suitability: Not suitable'.
-Step 5: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Oct 2027, 09:00–17:00. It was not changed or cancelled.</t>
+          <t>Step 1: The 'SPM68 Outgrown Room' item shows 'Flagged because: the expected attendance changed', 'Suitability: Not suitable' with 'Theatre capacity is 100 - your event expects 150.', 'Availability: Available' and 'This booking can't be kept while it doesn't meet the event's requirements.' It has no 'Keep booking' button. It still has 'Find a replacement venue' and 'Open Venue tab'.
+Step 2: The 'SPM68 Outgrown Room' item is still listed, still with 'Suitability: Not suitable' and no 'Keep booking' button.
+Step 3: The event's Venue tab opens. Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Oct 2027, 09:00–17:00. It was not changed or cancelled.</t>
         </is>
       </c>
     </row>
@@ -4181,7 +3983,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Flagged bookings at a blocked venue and at a retired venue are shown as not available with the reason, and neither can be kept</t>
+          <t>Flagged bookings at a blocked venue and at a retired venue are shown as not available with the reason, and neither is offered 'Keep booking'</t>
         </is>
       </c>
     </row>
@@ -4193,11 +3995,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Venue Trouble Day' is in Planning, assigned to Daniel Tan, on 9 Oct 2027, 09:00-17:00, for 40 people in Theatre layout. It has two approved venue bookings, both flagged: SPM68 Closed Room, which Venue Staff marked unavailable for maintenance from 9 Oct 2027, 08:00 to 9 Oct 2027, 18:00; and SPM68 Retired Room, which has been retired. Logged in as Daniel Tan. Keeping is refused in this case, so nothing is changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="98.5" customHeight="1">
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Venue Trouble Day' is in Planning, assigned to Daniel Tan, on 9 Oct 2027, 09:00-17:00, for 40 people in Theatre layout. It has two approved venue bookings, both flagged: SPM68 Closed Room, which Venue Staff marked unavailable for maintenance from 9 Oct 2027, 08:00 to 9 Oct 2027, 18:00; and SPM68 Retired Room, which has been retired. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4206,10 +4008,7 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
-2. Click 'Keep booking' in the 'SPM68 Venue Trouble Day' item for SPM68 Closed Room
-3. Click 'Keep booking' in the 'SPM68 Venue Trouble Day' item for SPM68 Retired Room
-4. Click 'SPM68 Venue Trouble Day' in either item
-5. Click the 'Venue' tab</t>
+2. Click 'Open Venue tab' in either 'SPM68 Venue Trouble Day' item</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4026,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="274" customHeight="1">
+    <row r="7" ht="220" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4235,10 +4034,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: Two separate items are listed for 'SPM68 Venue Trouble Day'. The SPM68 Closed Room item shows 'Flagged because: the venue is unavailable during this booking', 'Suitability: Suitable' and 'Availability: Not available' with 'SPM68 Closed Room is unavailable at this time (maintenance, 9 Oct 2027, 08:00–18:00).' The SPM68 Retired Room item shows 'Flagged because: the venue has been retired' and 'Availability: Not available' with 'SPM68 Retired Room has been retired.'
-Step 2: The flag is NOT cleared. The message 'SPM68 Closed Room no longer meets this event's requirements: SPM68 Closed Room is unavailable at this time (maintenance, 9 Oct 2027, 08:00–18:00).' is shown in that item, and the item is still listed.
-Step 3: The flag is NOT cleared. The message 'SPM68 Retired Room no longer meets this event's requirements: SPM68 Retired Room has been retired.' is shown in that item, and the item is still listed.
-Step 5: Under 'Booking requests', SPM68 Closed Room and SPM68 Retired Room are both still listed as 'Approved' for 9 Oct 2027, 09:00–17:00. Neither was changed or cancelled.</t>
+          <t>Step 1: Two separate items are listed for 'SPM68 Venue Trouble Day'. The SPM68 Closed Room item shows 'Flagged because: the venue is unavailable during this booking', 'Suitability: Suitable' and 'Availability: Not available' with 'SPM68 Closed Room is unavailable at this time (maintenance, 9 Oct 2027, 08:00–18:00).' The SPM68 Retired Room item shows 'Flagged because: the venue has been retired' and 'Availability: Not available' with 'SPM68 Retired Room has been retired.' Each item shows 'This booking can't be kept while it doesn't meet the event's requirements.' and has no 'Keep booking' button; each still has 'Find a replacement venue' and 'Open Venue tab'.
+Step 2: The event's Venue tab opens. Under 'Booking requests', SPM68 Closed Room and SPM68 Retired Room are both still listed as 'Approved' for 9 Oct 2027, 09:00–17:00. Neither was changed or cancelled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-68: keep from the Readiness tab; closed events and waived items
- The Readiness tab's flagged booking and equipment rows give the
  assigned coordinator Keep booking / Keep reservation, under the same
  rule as the Flagged Arrangements page (only while it still meets the
  event's requirements), and a Review in Flagged Arrangements link. The
  tab reads the same live result as the page, so the two never disagree.
  GET /api/events/[id]/arrangements adds canReviewFlags.
- Flagged Arrangements leaves out events that are completed, cancelled,
  rejected or withdrawn.
- A flagged arrangement marked as not required is still listed, and
  says so: waiving it does not clear the flag.
- Manual cases 14 -> 15: TC05 keeps from Readiness, TC06 checks Readiness
  offers no Keep for a room that is too small, TC15 covers the two edge
  cases. Two fixture events added for it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-68_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-68_Test_Cases.xlsx
@@ -22,6 +22,7 @@
     <sheet name="TC12" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -461,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -661,7 +662,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>A flagged venue booking blocks confirmation until it is kept; keeping one that still meets the event's requirements clears the flag and leaves the booking unchanged</t>
+          <t>A flagged venue booking blocks confirmation until it is kept; keeping it from the event's Readiness tab clears the flag, takes it off the Flagged Arrangements page and leaves the booking unchanged</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -693,7 +694,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking': the unmet requirement is named, the flag stays and the booking is unchanged</t>
+          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking' on the Flagged Arrangements page or on the event's Readiness tab: the unmet requirement is named, the flag stays and the booking is unchanged</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -968,63 +969,96 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC15</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC15</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>A flagged booking that was marked as not required is still listed and says so, and a flagged booking on a cancelled event is not listed</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>AC1, AC15</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
         </is>
       </c>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="9" t="n"/>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="71.5" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC02
 SPM-68-TC03
-SPM-68-TC04</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+SPM-68-TC04
+SPM-68-TC15</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Each flagged arrangement shows the event, the arrangement, and why it was flagged (e.g. event date changed, attendance changed, venue attributes updated, venue setup or turnaround time changed, venue retired, venue blocked, equipment marked unavailable).</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC07
@@ -1032,42 +1066,42 @@
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="31" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="31" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Given an event has more than one venue booking, when one of them is flagged, then only the flagged booking is listed.</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="71.5" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC01</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="71.5" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC05
@@ -1076,65 +1110,65 @@
 SPM-68-TC08</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="44.5" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="44.5" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>For a flagged equipment reservation, the current availability result for the event's present dates and quantities is shown.</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC09
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="44.5" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="44.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>AC6</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Given the arrangement still meets the event's requirements, when the Coordinator keeps it, then the flag is cleared and the arrangement is unchanged.</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC05
-SPM-68-TC09</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="58" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC05
+SPM-68-TC09</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC06
 SPM-68-TC07
@@ -1142,119 +1176,98 @@
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="71.5" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="71.5" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>AC8</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>For flagged registrations, the number of attendees registered or on the waiting list is shown, with why they were flagged: the event's date or time changed (see: Update Event Information, SPM-62), or the registration capacity was lowered below the number registered or registration was turned off (see: Configure Event Registration, SPM-64).</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01
-SPM-68-TC11</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="31" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>AC9</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC11</t>
+          <t>SPM-68-TC01
+SPM-68-TC11</t>
         </is>
       </c>
       <c r="F29" s="9" t="n"/>
     </row>
-    <row r="30" ht="17.5" customHeight="1">
+    <row r="30" ht="31" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>AC10</t>
+          <t>AC9</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Flagged registrations do not prevent confirmation.</t>
+          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC12</t>
+          <t>SPM-68-TC11</t>
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
     </row>
-    <row r="31" ht="58" customHeight="1">
+    <row r="31" ht="17.5" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC10</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
+          <t>Flagged registrations do not prevent confirmation.</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13</t>
+          <t>SPM-68-TC12</t>
         </is>
       </c>
       <c r="F31" s="9" t="n"/>
     </row>
-    <row r="32" ht="44.5" customHeight="1">
+    <row r="32" ht="58" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC11</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
+          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13
-SPM-68-TC14</t>
+          <t>SPM-68-TC13</t>
         </is>
       </c>
       <c r="F32" s="9" t="n"/>
     </row>
-    <row r="33" ht="31" customHeight="1">
+    <row r="33" ht="44.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC12</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Replacing a venue does not change the event's own information or status.</t>
+          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
@@ -1267,20 +1280,41 @@
       </c>
       <c r="F33" s="9" t="n"/>
     </row>
-    <row r="34" ht="98.5" customHeight="1">
+    <row r="34" ht="31" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>AC14</t>
+          <t>AC13</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+          <t>Replacing a venue does not change the event's own information or status.</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC13
+SPM-68-TC14</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="98.5" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>AC14</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC05
 SPM-68-TC06
@@ -1291,62 +1325,65 @@
 SPM-68-TC14</t>
         </is>
       </c>
-      <c r="F34" s="9" t="n"/>
-    </row>
-    <row r="35" ht="44.5" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="F35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="44.5" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>AC15</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>A flagged venue booking or equipment reservation counts as outstanding and prevents confirmation until it is resolved (see: Track Outstanding Arrangements).</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC05</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="31" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>AC16</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
         </is>
       </c>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="11" t="inlineStr">
         <is>
+          <t>SPM-68-TC05
+SPM-68-TC15</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="31" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>AC16</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
           <t>SPM-68-TC02</t>
         </is>
       </c>
-      <c r="F36" s="9" t="n"/>
-    </row>
-    <row r="38" ht="260.5" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="F37" s="9" t="n"/>
+    </row>
+    <row r="39" ht="287.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>prisma/schema.prisma
 prisma/seed.ts
 scripts/seed-spm68.ts
+src/app/api/events/[id]/arrangements/route.ts
 src/app/api/events/[id]/venue-bookings/[bookingId]/route.ts
 src/app/api/flagged-arrangements/route.ts
 src/app/events/[id]/booking/new/page.tsx
+src/app/events/[id]/readiness/page.tsx
 src/app/events/[id]/venue/page.tsx
 src/app/flagged/page.tsx
 src/app/venues/search/page.tsx
@@ -1362,10 +1399,10 @@
 src/lib/venueSuitability.ts</t>
         </is>
       </c>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="8" t="n"/>
-      <c r="E38" s="8" t="n"/>
-      <c r="F38" s="9" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="36">
@@ -1377,19 +1414,18 @@
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B37:D37"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="E31:F31"/>
-    <mergeCell ref="B20:D20"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="B38:F38"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B26:D26"/>
@@ -1402,6 +1438,7 @@
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E37:F37"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E21:F21"/>
@@ -1421,6 +1458,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2675,13 +2713,186 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-68-TC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A flagged booking that was marked as not required is still listed and says so, and a flagged booking on a cancelled event is not listed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>The SPM-68 fixtures are loaded (npm run fixtures:spm68). 'SPM68 Waived Room' is in Planning, assigned to Daniel Tan, on 23 Oct 2027, 09:00-17:00, for 40 people in Theatre layout; its approved booking at SPM68 Annex is flagged because the expected attendance changed, and Daniel Tan marked it as not required. 'SPM68 Cancelled Day' is Cancelled, assigned to Daniel Tan, on 24 Oct 2027, with an approved booking at SPM68 Annex that is also flagged. Logged in as Daniel Tan. Nothing is changed in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Flagged Arrangements' in the sidebar
+2. Click 'SPM68 Waived Room' in its item
+3. Click the 'Readiness' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>SPM68 Waived Room (Planning): SPM68 Annex, Approved, flagged, marked as not required
+SPM68 Cancelled Day (Cancelled): SPM68 Annex, Approved, flagged</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: On the 'Venue bookings' tab there is an item for 'SPM68 Waived Room' showing 'SPM68 Annex (SPM68-ANX)', 'Flagged because: the expected attendance changed', 'Marked as not required for this event, so it does not block confirmation.', 'Suitability: Suitable' and 'Availability: Available', with a 'Keep booking' button. There is no item for 'SPM68 Cancelled Day'.
+Step 3: 'SPM68 Annex' shows 'Approved' and 'Not required'. It still has the link 'Review in Flagged Arrangements' and a 'Keep booking' button, beside 'Mark as required'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2870,6 +3081,28 @@
         </is>
       </c>
       <c r="C16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="179.5" customHeight="1">
+      <c r="A17" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-13 (Kristen), replacing the earlier decision that the Readiness tab only links: a flagged booking or equipment line on the event's Readiness tab (Track Outstanding Arrangements, SPM-33) has the same 'Keep booking' / 'Keep reservation' as the Flagged Arrangements page, under the same rule - only while it still meets the event's requirements; otherwise the row lists what is unmet and says it can't be kept. The result is the one the Flagged Arrangements page shows (the same request), so the two screens never disagree. The row also has 'Review in Flagged Arrangements', a link to the matching tab, which is where a replacement is searched for. Only the assigned Coordinator sees either, at any event status; another Coordinator reading the tab sees neither (AC16). After keeping, the tab says 'Flag cleared' with '&lt;arrangement&gt; was kept as it is.' (SPM-68-TC05, SPM-68-TC06).</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="152.5" customHeight="1">
+      <c r="A18" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-13 (Kristen): two cases the criteria do not mention. (1) An event that is Completed, Cancelled, Rejected or Withdrawn is left out of the Flagged Arrangements page: there is nothing left for its flags to go wrong with. (2) A flagged booking or equipment line that was marked as not required on the Readiness tab stops blocking confirmation, but that waives it rather than resolving the flag, so it is still listed (AC1) with 'Marked as not required for this event, so it does not block confirmation.' and can still be kept; the Readiness tab keeps its link and Keep button on it too (SPM-68-TC15). The fixtures add 'SPM68 Waived Room' (23 Oct) and 'SPM68 Cancelled Day' (24 Oct), 13 events in all.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3619,7 +3852,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -3627,7 +3860,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A flagged venue booking blocks confirmation until it is kept; keeping one that still meets the event's requirements clears the flag and leaves the booking unchanged</t>
+          <t>A flagged venue booking blocks confirmation until it is kept; keeping it from the event's Readiness tab clears the flag, takes it off the Flagged Arrangements page and leaves the booking unchanged</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3887,12 @@
           <t>1. Click 'All Events' in the sidebar
 2. Click 'SPM68 Attendance Review' in the list
 3. Click the 'Readiness' tab
-4. Click 'Flagged Arrangements' in the sidebar
-5. Click 'Keep booking' in the 'SPM68 Attendance Review' item
-6. Click 'All Events' in the sidebar
-7. Click 'SPM68 Attendance Review' in the list
+4. Click 'Review in Flagged Arrangements' in the 'SPM68 Hall' item
+5. Click 'SPM68 Attendance Review' in its item
+6. Click the 'Readiness' tab
+7. Click 'Keep booking' in the 'SPM68 Hall' item
 8. Click the 'Venue' tab
-9. Click the 'Readiness' tab</t>
+9. Click 'Flagged Arrangements' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3909,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="233.5" customHeight="1">
+    <row r="7" ht="274" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3684,11 +3917,11 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: 'SPM68 Hall' shows 'Approved' and 'Outstanding', and says it is flagged for review: the expected attendance changed. The message '1 arrangement still blocks confirmation' is shown.
-Step 4: On the 'Venue bookings' tab, the 'SPM68 Attendance Review' item shows 'SPM68 Hall (SPM68-HAL)', 'Flagged because: the expected attendance changed', 'Suitability: Suitable' and 'Availability: Available'.
-Step 5: The message 'Flag cleared' is shown with 'SPM68 Hall for SPM68 Attendance Review was kept as it is.' The 'SPM68 Attendance Review' item is no longer listed.
+          <t>Step 3: 'SPM68 Hall' shows 'Approved' and 'Outstanding', and says it is flagged for review: the expected attendance changed. It has the link 'Review in Flagged Arrangements' and the buttons 'Keep booking' and 'Mark as not required'. The message '1 arrangement still blocks confirmation' is shown.
+Step 4: The 'Flagged Arrangements' page opens on the 'Venue bookings' tab, where the 'SPM68 Attendance Review' item shows 'SPM68 Hall (SPM68-HAL)', 'Flagged because: the expected attendance changed', 'Suitability: Suitable' and 'Availability: Available', with a 'Keep booking' button.
+Step 7: The message 'Flag cleared' is shown with 'SPM68 Hall was kept as it is.' 'SPM68 Hall' now shows 'Approved' and 'Complete', with no mention of being flagged, no 'Keep booking' button and no 'Review in Flagged Arrangements' link. The message 'Nothing is blocking confirmation' is shown.
 Step 8: Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 6 Oct 2027, 09:00–17:00 in Theatre layout. Its venue, times, layout and status are unchanged.
-Step 9: 'SPM68 Hall' shows 'Approved' and 'Complete', with no mention of being flagged. The message 'Nothing is blocking confirmation' is shown.</t>
+Step 9: On the 'Venue bookings' tab there is no longer an item for 'SPM68 Attendance Review'.</t>
         </is>
       </c>
     </row>
@@ -3801,7 +4034,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -3809,7 +4042,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking': the unmet requirement is named, the flag stays and the booking is unchanged</t>
+          <t>A flagged venue booking whose room is now too small is not offered 'Keep booking' on the Flagged Arrangements page or on the event's Readiness tab: the unmet requirement is named, the flag stays and the booking is unchanged</t>
         </is>
       </c>
     </row>
@@ -3825,7 +4058,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44.5" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3835,7 +4068,8 @@
         <is>
           <t>1. Click 'Flagged Arrangements' in the sidebar
 2. Refresh the page in the browser
-3. Click 'Open Venue tab' in the 'SPM68 Outgrown Room' item</t>
+3. Click 'Open Venue tab' in the 'SPM68 Outgrown Room' item
+4. Click the 'Readiness' tab</t>
         </is>
       </c>
     </row>
@@ -3852,7 +4086,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="179.5" customHeight="1">
+    <row r="7" ht="247" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3862,7 +4096,8 @@
         <is>
           <t>Step 1: The 'SPM68 Outgrown Room' item shows 'Flagged because: the expected attendance changed', 'Suitability: Not suitable' with 'Theatre capacity is 100 - your event expects 150.', 'Availability: Available' and 'This booking can't be kept while it doesn't meet the event's requirements.' It has no 'Keep booking' button. It still has 'Find a replacement venue' and 'Open Venue tab'.
 Step 2: The 'SPM68 Outgrown Room' item is still listed, still with 'Suitability: Not suitable' and no 'Keep booking' button.
-Step 3: The event's Venue tab opens. Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Oct 2027, 09:00–17:00. It was not changed or cancelled.</t>
+Step 3: The event's Venue tab opens. Under 'Booking requests', SPM68 Hall is still listed as 'Approved' for 8 Oct 2027, 09:00–17:00. It was not changed or cancelled.
+Step 4: 'SPM68 Hall' shows 'Approved' and 'Outstanding', with 'Theatre capacity is 100 - your event expects 150.' and 'This booking can't be kept while it doesn't meet the event's requirements.' It has the link 'Review in Flagged Arrangements' and no 'Keep booking' button.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-68: Keep refuses what the list would never show; TC13/TC14 fixed
- POST /api/flagged-arrangements now applies the same limits GET lists
  by: 400 for an event that is completed, cancelled, rejected or
  withdrawn (all three kinds), for a booking that is not pending or
  approved, and for an equipment request that is cancelled or could not
  be provided. A direct request can no longer clear those flags.
- SPM-68-TC13's last step and TC14's first step no longer list
  'Keep booking' on the Outgrown Room's Hall booking, which does not fit.
- docs/PERMISSIONS.md and the changelog entry list the new refusals.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-68_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-68_Test_Cases.xlsx
@@ -2435,7 +2435,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="328" customHeight="1">
+    <row r="7" ht="368.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2448,7 +2448,7 @@
 Step 4: The message 'Booking request sent to Venue Staff.' is shown.
 Step 5: Under 'Booking requests', SPM68 Spare Room is listed as 'Pending' and SPM68 Hall is still listed as 'Approved', both for 8 Oct 2027, 09:00–17:00.
 Step 6: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
-Step 7: The 'SPM68 Outgrown Room' item for SPM68 Hall is still listed on the 'Venue bookings' tab, still flagged, with 'Keep booking', 'Find a replacement venue' and 'Open Venue tab'.</t>
+Step 7: The 'SPM68 Outgrown Room' item for SPM68 Hall is still listed on the 'Venue bookings' tab, still flagged, with 'Suitability: Not suitable', 'This booking can't be kept while it doesn't meet the event's requirements.' and the buttons 'Find a replacement venue' and 'Open Venue tab'. It has no 'Keep booking' button: requesting a replacement does not make the room big enough.</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'SPM68 Outgrown Room' item for SPM68 Hall is listed with 'Keep booking', 'Find a replacement venue' and 'Open Venue tab'. It has no 'Release booking' or 'Withdraw request' button.
+          <t>Step 1: The 'SPM68 Outgrown Room' item for SPM68 Hall is listed with 'Find a replacement venue' and 'Open Venue tab'. It has no 'Keep booking' button, because the room no longer fits, and no 'Release booking' or 'Withdraw request' button.
 Step 2: The event's Venue tab opens. Under 'Booking requests', SPM68 Hall is 'Approved' with a 'Release booking' button and SPM68 Spare Room is 'Pending'.
 Step 3: A dialog 'Release this booking?' reads 'SPM68 Hall (SPM68-HAL) on 8 Oct 2027, 09:00–17:00 will be freed for other events, and Venue Staff will be notified.'
 Step 5: The dialog closes. The message 'Booking released' is shown. SPM68 Hall is still listed, now as 'Released' with 'Reason for release: Room is too small for 150 people.' and no button. SPM68 Spare Room is still 'Pending' for 8 Oct 2027, 09:00–17:00.

</xml_diff>

<commit_message>
SPM-68: judge each flagged booking against its own space (SPM-90)
- A flagged booking is re-checked against the space it is for. The main
  programme (SPM-90's default purpose, or none on a booking made before
  SPM-90) follows the event's present attendance and layout; any other
  space, e.g. a breakout room, is held to its own as booked. spaceNeeds()
  in src/lib/flaggedArrangements.ts. Items show "Space: <purpose>".
- Find a replacement venue fills the search the same way, and Request
  booking carries the space along (purpose, attendance, layout). The
  request form now reads purpose from its address, as it did attendance
  and layout - without it a replacement request was refused for having
  no purpose.
- Manual cases 15 -> 16: TC13 Step 3 expects the space filled in; TC16
  covers a main room and a breakout room after the event grew. All
  passed by hand. Fixture event 'SPM68 Breakout Growth' added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-68_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-68_Test_Cases.xlsx
@@ -23,6 +23,7 @@
     <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1001,40 +1002,72 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC16</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>When an event grows, its main programme room is held to the event's new attendance and cannot be kept, while its breakout room is held to its own attendance and can be kept</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>AC4, AC6, AC7</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="71.5" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
         </is>
       </c>
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="71.5" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can view a list of flagged venue bookings, equipment reservations and registrations for the events assigned to them.</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC02
@@ -1043,22 +1076,22 @@
 SPM-68-TC15</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Each flagged arrangement shows the event, the arrangement, and why it was flagged (e.g. event date changed, attendance changed, venue attributes updated, venue setup or turnaround time changed, venue retired, venue blocked, equipment marked unavailable).</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC07
@@ -1066,229 +1099,211 @@
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="31" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="31" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Given an event has more than one venue booking, when one of them is flagged, then only the flagged booking is listed.</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="71.5" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
         </is>
       </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC01</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="85" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>For a flagged venue booking, the current suitability and availability result for the event's present requirements is shown.</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC05
 SPM-68-TC06
 SPM-68-TC07
-SPM-68-TC08</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="44.5" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+SPM-68-TC08
+SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="44.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>For a flagged equipment reservation, the current availability result for the event's present dates and quantities is shown.</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC01
 SPM-68-TC09
 SPM-68-TC10</t>
         </is>
       </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="44.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="44.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>AC6</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Given the arrangement still meets the event's requirements, when the Coordinator keeps it, then the flag is cleared and the arrangement is unchanged.</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC05
-SPM-68-TC09</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
         </is>
       </c>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
+          <t>SPM-68-TC05
+SPM-68-TC09
+SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="71.5" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Given the arrangement no longer meets the event's requirements, when the Coordinator attempts to keep it, then the flag is not cleared and the unmet requirement is identified.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
           <t>SPM-68-TC06
 SPM-68-TC07
 SPM-68-TC08
-SPM-68-TC10</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="71.5" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+SPM-68-TC10
+SPM-68-TC16</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="71.5" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>AC8</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>For flagged registrations, the number of attendees registered or on the waiting list is shown, with why they were flagged: the event's date or time changed (see: Update Event Information, SPM-62), or the registration capacity was lowered below the number registered or registration was turned off (see: Configure Event Registration, SPM-64).</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC01
-SPM-68-TC11</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n"/>
-    </row>
-    <row r="30" ht="31" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>AC9</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC11</t>
+          <t>SPM-68-TC01
+SPM-68-TC11</t>
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
     </row>
-    <row r="31" ht="17.5" customHeight="1">
+    <row r="31" ht="31" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>AC10</t>
+          <t>AC9</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Flagged registrations do not prevent confirmation.</t>
+          <t>Given registrations are flagged, when the Coordinator marks them as reviewed, then the flag is cleared and no registration is changed.</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC12</t>
+          <t>SPM-68-TC11</t>
         </is>
       </c>
       <c r="F31" s="9" t="n"/>
     </row>
-    <row r="32" ht="58" customHeight="1">
+    <row r="32" ht="17.5" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC10</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
+          <t>Flagged registrations do not prevent confirmation.</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13</t>
+          <t>SPM-68-TC12</t>
         </is>
       </c>
       <c r="F32" s="9" t="n"/>
     </row>
-    <row r="33" ht="44.5" customHeight="1">
+    <row r="33" ht="58" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC11</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
+          <t>From a flagged venue booking, the Coordinator can search for a replacement venue, with the search pre-filled from that booking's date, start and end times, attendance, layout, accessibility and facility requirements.</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>SPM-68-TC13
-SPM-68-TC14</t>
+          <t>SPM-68-TC13</t>
         </is>
       </c>
       <c r="F33" s="9" t="n"/>
     </row>
-    <row r="34" ht="31" customHeight="1">
+    <row r="34" ht="44.5" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC12</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Replacing a venue does not change the event's own information or status.</t>
+          <t>The Coordinator can request the replacement venue; the flagged booking stays on the event record until the Coordinator releases it (see: Withdraw or Release Venue Booking).</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
@@ -1301,20 +1316,41 @@
       </c>
       <c r="F34" s="9" t="n"/>
     </row>
-    <row r="35" ht="98.5" customHeight="1">
+    <row r="35" ht="31" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>AC14</t>
+          <t>AC13</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+          <t>Replacing a venue does not change the event's own information or status.</t>
         </is>
       </c>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>SPM-68-TC13
+SPM-68-TC14</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="98.5" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>AC14</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>A flagged arrangement is never changed or cancelled automatically.</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>SPM-68-TC05
 SPM-68-TC06
@@ -1325,56 +1361,56 @@
 SPM-68-TC14</t>
         </is>
       </c>
-      <c r="F35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="44.5" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="F36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="44.5" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>AC15</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>A flagged venue booking or equipment reservation counts as outstanding and prevents confirmation until it is resolved (see: Track Outstanding Arrangements).</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="11" t="inlineStr">
-        <is>
-          <t>SPM-68-TC05
-SPM-68-TC15</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n"/>
-    </row>
-    <row r="37" ht="31" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>AC16</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
         </is>
       </c>
       <c r="C37" s="8" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="11" t="inlineStr">
         <is>
+          <t>SPM-68-TC05
+SPM-68-TC15</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="31" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>AC16</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>A Coordinator does not see flagged arrangements for events assigned to other Coordinators.</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
           <t>SPM-68-TC02</t>
         </is>
       </c>
-      <c r="F37" s="9" t="n"/>
-    </row>
-    <row r="39" ht="287.5" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="F38" s="9" t="n"/>
+    </row>
+    <row r="40" ht="287.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>prisma/schema.prisma
 prisma/seed.ts
@@ -1399,10 +1435,10 @@
 src/lib/venueSuitability.ts</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="9" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="36">
@@ -1411,11 +1447,12 @@
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B38:D38"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E35:F35"/>
-    <mergeCell ref="B39:F39"/>
     <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="B30:D30"/>
@@ -1433,6 +1470,7 @@
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E25:F25"/>
@@ -1440,8 +1478,6 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1459,6 +1495,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2435,7 +2472,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="368.5" customHeight="1">
+    <row r="7" ht="395.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2444,7 +2481,7 @@
       <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The 'Find a venue' page opens, saying 'Filled in from the flagged booking at SPM68 Hall. Change any filter and search again.' 'From' reads 8 Oct 2027, 09:00 and 'To' reads 8 Oct 2027, 17:00. 'Expected attendance' reads 150. 'Room layout' reads 'Theatre'. 'Step-free access' is ticked under 'Accessibility requirements' and 'Fixed ceiling projector' is ticked under 'Required facilities'; nothing else is ticked. The results include 'SPM68 Spare Room (SPM68-SPR)' with a 'Request booking' button, and do not include SPM68 Hall.
-Step 3: The 'Request a venue booking' page opens for SPM68 Spare Room, with Date 8 Oct 2027, Start time 09:00 and End time 17:00 filled in.
+Step 3: The 'Request a venue booking' page opens for SPM68 Spare Room, with Date 8 Oct 2027, Start time 09:00 and End time 17:00, 'What is this space for?' reading 'Main programme', 'Expected attendance for this space' reading 150 and 'Room layout' reading 'Theatre', all filled in.
 Step 4: The message 'Booking request sent to Venue Staff.' is shown.
 Step 5: Under 'Booking requests', SPM68 Spare Room is listed as 'Pending' and SPM68 Hall is still listed as 'Approved', both for 8 Oct 2027, 09:00–17:00.
 Step 6: The status badge still reads 'Planning'. The event still shows 8 Oct 2027, 09:00–17:00, an expected attendance of 150 and Theatre layout.
@@ -2886,13 +2923,189 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-68-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>When an event grows, its main programme room is held to the event's new attendance and cannot be kept, while its breakout room is held to its own attendance and can be kept</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm68 before and after this case. 'SPM68 Breakout Growth' is in Planning, assigned to Daniel Tan, on 25 Oct 2027, 09:00-17:00, and now expects 150 people (it expected 80 when its rooms were booked). It has two approved bookings, both flagged because the expected attendance changed: SPM68 Hall for the 'Main programme' (Theatre seats 100, booked for 80) and SPM68 Annex for a 'Breakout room' (Theatre seats 60, booked for 40). Logged in as Daniel Tan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Flagged Arrangements' in the sidebar
+2. Click 'Keep booking' in the 'SPM68 Breakout Growth' item for SPM68 Annex
+3. Click 'SPM68 Breakout Growth' in the item that is left
+4. Click the 'Venue' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM68 Breakout Growth (Planning), 25 Oct 2027, 09:00-17:00, now 150 people
+SPM68 Hall: Main programme, booked for 80, Theatre seats 100 (flagged)
+SPM68 Annex: Breakout room, booked for 40, Theatre seats 60 (flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: Two items are listed for 'SPM68 Breakout Growth', each with 'Flagged because: the expected attendance changed'. The SPM68 Hall item shows 'Space: Main programme', 'Suitability: Not suitable' with 'Theatre capacity is 100 - this space expects 150.' and 'This booking can't be kept while it doesn't meet the event's requirements.', and has no 'Keep booking' button. The SPM68 Annex item shows 'Space: Breakout room', 'Suitability: Suitable' and 'Availability: Available', with a 'Keep booking' button.
+Step 2: The message 'Flag cleared' is shown with 'SPM68 Annex for SPM68 Breakout Growth was kept as it is.' The SPM68 Annex item is no longer listed; the SPM68 Hall item is still listed.
+Step 4: Under 'Booking requests', SPM68 Hall and SPM68 Annex are both still listed as 'Approved' for 25 Oct 2027, 09:00–17:00. Neither was changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2917,13 +3130,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="71.5" customHeight="1">
+    <row r="2" ht="85" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written before the code (TDD, 2026-10-13); the code was built to these cases and the automated tests the same day. All 15 cases were run by hand against the fixtures (npm run fixtures:spm68) on 2026-10-13 by Kristen, and all passed. Entries marked DECIDED were chosen here rather than taken from the story; change them in code and cases together.</t>
+          <t>Written before the code (TDD, 2026-10-13); the code was built to these cases and the automated tests the same day. All cases were run by hand against the fixtures (npm run fixtures:spm68) by Kristen and passed: TC01-TC15 on 2026-10-13, and TC13 (changed for SPM-90) and the new TC16 on 2026-10-15. Entries marked DECIDED were chosen here rather than taken from the story; change them in code and cases together.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
@@ -2989,7 +3202,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-13: what 'still meets the event's requirements' means for a venue booking (AC4, AC6, AC7). Suitability is the existing check (SPM-41) for the event's present attendance, layout and mandatory facilities - the session's attendance and layout for a session's booking. Availability is: the venue has not been retired; the booking's own times still cover the event's (or session's) present time, the rule a new request must pass (SPM-93); and nothing else holds or blocks the room for the booking's occupied time (the existing conflict check, SPM-44: an unavailable period, or another event's approved booking). Keep is refused unless both pass (SPM-68-TC06 to SPM-68-TC08).</t>
+          <t>DECIDED 2026-10-13: what 'still meets the event's requirements' means for a venue booking (AC4, AC6, AC7). Suitability is the existing check (SPM-41) for the attendance and layout of the space the booking is for (see the SPM-90 decision below) and the event's mandatory facilities. Availability is: the venue has not been retired; the booking's own times still cover the event's (or session's) present time, the rule a new request must pass (SPM-93); and nothing else holds or blocks the room for the booking's occupied time (the existing conflict check, SPM-44: an unavailable period, or another event's approved booking). Keep is refused unless both pass (SPM-68-TC06 to SPM-68-TC08).</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
@@ -3103,6 +3316,28 @@
         </is>
       </c>
       <c r="C18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="233.5" customHeight="1">
+      <c r="A19" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-15 (Kristen), after Check Each Venue Against Its Own Requirements (SPM-90) reached main: since SPM-90 a booking is for a space, with its own purpose, attendance and layout, copied from the event when it was requested unless the Coordinator set them. A flagged booking is re-checked against its space as it is now. The main programme - a booking whose purpose is SPM-90's default 'Main programme' (which the request form gives an event's first room), or that has none because it was made before SPM-90 - is the event's own room and follows the event: its present attendance and layout, or the session's. Any other space, e.g. 'Breakout room', is held to its own attendance and layout as booked, so an event that grew does not make a breakout room too small for its own number. The item shows 'Space: &lt;purpose&gt;', and 'Find a replacement venue' fills the search the same way (SPM-68-TC16). Limitation: a main room the Coordinator named something other than 'Main programme' (e.g. 'Plenary') is held to its own booked attendance, so an event that grew does not make it fail; the Coordinator has to judge it from the flag reason.</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="139" customHeight="1">
+      <c r="A20" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-15 (Kristen), found while re-running the cases after SPM-90 reached main: since SPM-90 a request must say what its space is for, and the request form fills in 'Main programme' only for an event's first room. A replacement is requested while the flagged booking still stands, so the box started empty and TC13's 'Submit request' was refused. 'Request booking' from a replacement search now carries the space along: what the flagged booking was for ('Main programme' for one made before spaces were named), and the attendance and layout searched for. The request form takes 'purpose' from its address as it already took 'attendance' and 'layout' (SPM-68-TC13).</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>